<commit_message>
vault backup: 2026-07-16 15:40:31
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/MVP功能清单.xlsx
+++ b/公司项目/认知作战/文档/MVP功能清单.xlsx
@@ -5,6 +5,8 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="rId1"/>
     <x:sheet name="MVP范围总览" sheetId="2" r:id="R8e1c6d9b327041cc"/>
     <x:sheet name="MVP功能清单" sheetId="3" r:id="R9e45136bd8034e26"/>
+    <x:sheet name="阶段排期" sheetId="4" r:id="Rb46ec1a74f294565"/>
+    <x:sheet name="风险登记" sheetId="5" r:id="R195041dac57d4f4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -54,7 +56,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -71,6 +73,31 @@
         <x:fgColor rgb="FF1F4E79"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFC7CE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBDD7EE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFEB9C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9D9D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC6EFCE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -84,7 +111,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyFont="1" applyFill="1"/>
@@ -101,6 +128,30 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -220,6 +271,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" rgb="FF1F4E79"/>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="95" customWidth="1"/>
@@ -276,8 +331,11 @@
         <x:v>一、文档目的</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="60" customHeight="1">
       <x:c r="A10" s="5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="B10" s="8" t="str">
         <x:v>本清单是「认知作战平台」MVP（最小可行产品）版本的功能分解与交付规划。基于《MVP 版本规划》文档的决策结论，将 7 子系统 40 项需求裁剪为可演示的最小功能集，明确每项功能：是否纳入 MVP、优先级、所属子系统/模块/需求、降级路径（排期吃紧时先砍什么）。</x:v>
       </x:c>
     </x:row>
@@ -286,8 +344,11 @@
         <x:v>二、MVP 定位（决策结论）</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="42" customHeight="1">
+    <x:row r="13" ht="60" customHeight="1">
       <x:c r="A13" s="5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="B13" s="8" t="str">
         <x:v>① 目标=可演示的最小产品（重 UI/可见效果，非架构验证、非真实上线）；② 演示主线=智能体蜂群养号/发帖（一片真机同时在动 + 智能体看屏幕自主决策）；③ 子系统优先级=MC &gt; SWM &gt; IRS 主场，OCC/DC 闭环配角，OM/COM 底座；④ 时间/人力=3 个月 · 2-4 人；⑤ 交付物=可现场演示系统 + 说明文档。</x:v>
       </x:c>
     </x:row>
@@ -296,8 +357,11 @@
         <x:v>三、三个架构原则（MVP 必须保住）</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="42" customHeight="1">
+    <x:row r="16" ht="60" customHeight="1">
       <x:c r="A16" s="5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
         <x:v>CON-07 动作收口：所有真机动作经 MC 执行网关落地（可观测/可审计/可熔断）；CON-10 推理与执行分离：agent-runtime 调 IRS 视觉推理不经网关，产出的动作指令再经网关落地；CON-08 双执行模式：脚本模式保底（确定性流程）+ 智能体模式亮点（VLM 视觉决策）。</x:v>
       </x:c>
     </x:row>
@@ -306,8 +370,11 @@
         <x:v>四、优先级图例</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="42" customHeight="1">
+    <x:row r="19" ht="60" customHeight="1">
       <x:c r="A19" s="5" t="str">
+        <x:v/>
+      </x:c>
+      <x:c r="B19" s="8" t="str">
         <x:v>P0=演示灵魂，必须做（砍了演示垮）；P1=核心支撑，应该做；P2=配角/锦上添花，排期吃紧可砍。状态：MVP=纳入本版；降级=排期吃紧时按降级路径退而求其次；砍=本版不做。</x:v>
       </x:c>
     </x:row>
@@ -334,6 +401,9 @@
       <x:c r="B23" t="str">
         <x:v>7 子系统的 MVP 范围一览（做/降级/砍）、技术栈、演示角色</x:v>
       </x:c>
+      <x:c r="C23">
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
@@ -342,6 +412,9 @@
       <x:c r="B24" t="str">
         <x:v>逐条功能分解：子系统/模块/需求/功能点/优先级/状态/降级路径（核心表）</x:v>
       </x:c>
+      <x:c r="C24">
+        <x:v>27</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
@@ -350,6 +423,9 @@
       <x:c r="B25" t="str">
         <x:v>3 个月分阶段、里程碑、人力分配</x:v>
       </x:c>
+      <x:c r="C25">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
@@ -358,8 +434,12 @@
       <x:c r="B26" t="str">
         <x:v>两个高风险项 + 应对/降级路径</x:v>
       </x:c>
+      <x:c r="C26">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
+  <x:pageSetup fitToWidth="1" fitToHeight="1" orientation="landscape"/>
 </x:worksheet>
 </file>
 
@@ -367,6 +447,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF1F4E79"/>
+    <x:pageSetUpPr fitToPage="1"/>
   </x:sheetPr>
   <x:cols>
     <x:col min="1" max="1" width="20" customWidth="1"/>
@@ -568,11 +649,27 @@
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:pageSetup fitToWidth="1" fitToHeight="1" orientation="landscape"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFC00000"/>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
+  <x:cols>
+    <x:col min="1" max="1" width="8" customWidth="1"/>
+    <x:col min="2" max="2" width="8" customWidth="1"/>
+    <x:col min="3" max="3" width="12" customWidth="1"/>
+    <x:col min="4" max="4" width="14" customWidth="1"/>
+    <x:col min="5" max="5" width="58" customWidth="1"/>
+    <x:col min="6" max="6" width="8" customWidth="1"/>
+    <x:col min="7" max="7" width="8" customWidth="1"/>
+    <x:col min="8" max="8" width="42" customWidth="1"/>
+    <x:col min="9" max="9" width="26" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="6" t="str">
@@ -613,747 +710,1038 @@
         <x:v>备注</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" t="str">
         <x:v>MC-1</x:v>
       </x:c>
-      <x:c r="B4" t="str">
+      <x:c r="B4" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C4" t="str">
+      <x:c r="C4" s="8" t="str">
         <x:v>M-MC-01</x:v>
       </x:c>
-      <x:c r="D4" t="str">
+      <x:c r="D4" s="8" t="str">
         <x:v>R-MC-001</x:v>
       </x:c>
-      <x:c r="E4" t="str">
+      <x:c r="E4" s="8" t="str">
         <x:v>真机接入与台账：ADB/无障碍通道接入 3-8 台安卓真机；设备注册/台账/在线状态；Web 终端台账页(MC-02)</x:v>
       </x:c>
-      <x:c r="F4" t="str">
+      <x:c r="F4" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G4" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H4" t="str">
+      <x:c r="G4" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="str">
         <x:v>单类型真机即可，不接云手机/指纹浏览器</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5">
+      <x:c r="I4" s="8"/>
+    </x:row>
+    <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" t="str">
         <x:v>MC-2</x:v>
       </x:c>
-      <x:c r="B5" t="str">
+      <x:c r="B5" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C5" t="str">
+      <x:c r="C5" s="8" t="str">
         <x:v>M-MC-04</x:v>
       </x:c>
-      <x:c r="D5" t="str">
+      <x:c r="D5" s="8" t="str">
         <x:v>R-MC-004</x:v>
       </x:c>
-      <x:c r="E5" t="str">
+      <x:c r="E5" s="8" t="str">
         <x:v>mc-sfu 自建 mediasoup SFU：单设备实时控制(WebRTC) + 多终端宫格同屏预览</x:v>
       </x:c>
-      <x:c r="F5" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G5" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H5" t="str">
+      <x:c r="G5" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H5" s="8" t="str">
         <x:v>mc-sfu 故障→降级截图轮询；宫格可先做截图刷新</x:v>
       </x:c>
-      <x:c r="I5" t="str">
+      <x:c r="I5" s="8" t="str">
         <x:v>演示视觉灵魂：一片设备同时在动</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" t="str">
         <x:v>MC-3</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c r="B6" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C6" t="str">
+      <x:c r="C6" s="8" t="str">
         <x:v>M-MC-05</x:v>
       </x:c>
-      <x:c r="D6" t="str">
+      <x:c r="D6" s="8" t="str">
         <x:v>R-MC-005</x:v>
       </x:c>
-      <x:c r="E6" t="str">
+      <x:c r="E6" s="8" t="str">
         <x:v>统一执行网关：所有真机动作经网关落地，收口鉴权/记录/基础熔断；ADB/无障碍通道适配</x:v>
       </x:c>
-      <x:c r="F6" t="str">
+      <x:c r="F6" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G6" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H6" t="str">
+      <x:c r="G6" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H6" s="8" t="str">
         <x:v>熔断先做基础(失败计数)，不做全套规则</x:v>
       </x:c>
-      <x:c r="I6" t="str">
+      <x:c r="I6" s="8" t="str">
         <x:v>CON-07 动作收口，架构底线</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" t="str">
         <x:v>MC-4</x:v>
       </x:c>
-      <x:c r="B7" t="str">
+      <x:c r="B7" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C7" t="str">
+      <x:c r="C7" s="8" t="str">
         <x:v>M-MC-06</x:v>
       </x:c>
-      <x:c r="D7" t="str">
+      <x:c r="D7" s="8" t="str">
         <x:v>R-MC-006</x:v>
       </x:c>
-      <x:c r="E7" t="str">
+      <x:c r="E7" s="8" t="str">
         <x:v>双执行模式：脚本引擎(GraalVM JS 沙箱跑确定性流程) + agent-runtime(智能体运行时引擎)</x:v>
       </x:c>
-      <x:c r="F7" t="str">
+      <x:c r="F7" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G7" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H7" t="str">
+      <x:c r="G7" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H7" s="8" t="str">
         <x:v>智能体推理失败→agent-runtime 降级脚本(degrade_to_script)</x:v>
       </x:c>
-      <x:c r="I7" t="str">
+      <x:c r="I7" s="8" t="str">
         <x:v>CON-08 双执行模式，架构底线</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" t="str">
         <x:v>MC-5</x:v>
       </x:c>
-      <x:c r="B8" t="str">
+      <x:c r="B8" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C8" t="str">
+      <x:c r="C8" s="8" t="str">
         <x:v>M-MC-06</x:v>
       </x:c>
-      <x:c r="D8" t="str">
+      <x:c r="D8" s="8" t="str">
         <x:v>R-MC-006</x:v>
       </x:c>
-      <x:c r="E8" t="str">
+      <x:c r="E8" s="8" t="str">
         <x:v>agent-runtime：场景适配→读SWM记忆→调IRS多模态视觉推理→产出动作指令→经执行网关落地</x:v>
       </x:c>
-      <x:c r="F8" t="str">
+      <x:c r="F8" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G8" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H8" t="str">
+      <x:c r="G8" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H8" s="8" t="str">
         <x:v>VLM效果差→降级 UI树(a11y dump)+文本LLM；记忆不可用→无记忆运行</x:v>
       </x:c>
-      <x:c r="I8" t="str">
+      <x:c r="I8" s="8" t="str">
         <x:v>CON-10 推理执行分离；演示灵魂</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" t="str">
         <x:v>MC-6</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c r="B9" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C9" t="str">
+      <x:c r="C9" s="8" t="str">
         <x:v>M-MC-07</x:v>
       </x:c>
-      <x:c r="D9" t="str">
+      <x:c r="D9" s="8" t="str">
         <x:v>R-MC-007</x:v>
       </x:c>
-      <x:c r="E9" t="str">
+      <x:c r="E9" s="8" t="str">
         <x:v>任务管理：任务入队/分发/状态流转(简化状态机)；接收 OCC 编排下发与效果回传(II-10)</x:v>
       </x:c>
-      <x:c r="F9" t="str">
+      <x:c r="F9" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G9" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H9" t="str">
+      <x:c r="G9" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H9" s="8" t="str">
         <x:v>不做定时/重试/优先级全套</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10">
+      <x:c r="I9" s="8"/>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" t="str">
         <x:v>MC-7</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="B10" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C10" t="str">
+      <x:c r="C10" s="8" t="str">
         <x:v>M-MC-11</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="D10" s="8" t="str">
         <x:v>R-MC-011</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="E10" s="8" t="str">
         <x:v>账号主数据最小集：注册/凭据(AES-256-GCM加密)/平台/状态；作为账号权威源向SWM/OCC分发account_id</x:v>
       </x:c>
-      <x:c r="F10" t="str">
+      <x:c r="F10" s="13" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="G10" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H10" t="str">
+      <x:c r="G10" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H10" s="8" t="str">
         <x:v>不做风险评估/分类/完整生命周期</x:v>
       </x:c>
-      <x:c r="I10" t="str">
+      <x:c r="I10" s="8" t="str">
         <x:v>CON-11 账号权威源</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" t="str">
         <x:v>MC-8</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="B11" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C11" t="str">
+      <x:c r="C11" s="8" t="str">
         <x:v>M-MC-14</x:v>
       </x:c>
-      <x:c r="D11" t="str">
+      <x:c r="D11" s="8" t="str">
         <x:v>R-MC-014</x:v>
       </x:c>
-      <x:c r="E11" t="str">
+      <x:c r="E11" s="8" t="str">
         <x:v>智能体执行宿主：持存 SWM 同步的提示词包(agent_id主键)；执行前人设一致性校验；作为 OCC 智能体节点来源</x:v>
       </x:c>
-      <x:c r="F11" t="str">
+      <x:c r="F11" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G11" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H11" t="str">
+      <x:c r="G11" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H11" s="8" t="str">
         <x:v>人设校验可简化</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12">
+      <x:c r="I11" s="8"/>
+    </x:row>
+    <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" t="str">
         <x:v>MC-9</x:v>
       </x:c>
-      <x:c r="B12" t="str">
+      <x:c r="B12" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C12" t="str">
+      <x:c r="C12" s="8" t="str">
         <x:v>M-MC-01/04等</x:v>
       </x:c>
-      <x:c r="D12" t="str">
+      <x:c r="D12" s="8" t="str">
         <x:v>R-MC-002/003</x:v>
       </x:c>
-      <x:c r="E12" t="str">
+      <x:c r="E12" s="8" t="str">
         <x:v>代理 IP 绑定：真机一设备一账号一IP(简化版，固定代理IP)</x:v>
       </x:c>
-      <x:c r="F12" t="str">
+      <x:c r="F12" s="13" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="G12" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H12" t="str">
+      <x:c r="G12" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H12" s="8" t="str">
         <x:v>不做轮换/失效切换/代理池管理</x:v>
       </x:c>
-      <x:c r="I12" t="str">
+      <x:c r="I12" s="8" t="str">
         <x:v>CON-13 绑定规则</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" t="str">
         <x:v>MC-10</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B13" s="8" t="str">
         <x:v>MC</x:v>
       </x:c>
-      <x:c r="C13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="C13" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E13" s="8" t="str">
         <x:v>（砍）指纹浏览器/云手机/虚拟化真机/ARM板卡接入；完整账号生命周期；模板任务库；编排器MC-15；脚本IDE MC-16；熔断全套；录屏</x:v>
       </x:c>
       <x:c r="F13" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="G13" t="str">
+      <x:c r="G13" s="14" t="str">
         <x:v>砍</x:v>
       </x:c>
-      <x:c r="H13" t="str">
+      <x:c r="H13" s="8" t="str">
         <x:v>留 V1.1+</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14">
+      <x:c r="I13" s="8"/>
+    </x:row>
+    <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" t="str">
         <x:v>SWM-1</x:v>
       </x:c>
-      <x:c r="B14" t="str">
+      <x:c r="B14" s="8" t="str">
         <x:v>SWM</x:v>
       </x:c>
-      <x:c r="C14" t="str">
+      <x:c r="C14" s="8" t="str">
         <x:v>M-SWM-01</x:v>
       </x:c>
-      <x:c r="D14" t="str">
+      <x:c r="D14" s="8" t="str">
         <x:v>R-SWM-001</x:v>
       </x:c>
-      <x:c r="E14" t="str">
+      <x:c r="E14" s="8" t="str">
         <x:v>人设标签管理：Web 录入人设标签(身份/立场/语言风格)，挂 agent_id</x:v>
       </x:c>
-      <x:c r="F14" t="str">
+      <x:c r="F14" s="13" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="G14" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H14" t="str">
+      <x:c r="G14" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H14" s="8" t="str">
         <x:v>人工录入，不做自动生成</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15">
+      <x:c r="I14" s="8"/>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" t="str">
         <x:v>SWM-2</x:v>
       </x:c>
-      <x:c r="B15" t="str">
+      <x:c r="B15" s="8" t="str">
         <x:v>SWM</x:v>
       </x:c>
-      <x:c r="C15" t="str">
+      <x:c r="C15" s="8" t="str">
         <x:v>M-SWM-05</x:v>
       </x:c>
-      <x:c r="D15" t="str">
+      <x:c r="D15" s="8" t="str">
         <x:v>R-SWM-003</x:v>
       </x:c>
-      <x:c r="E15" t="str">
+      <x:c r="E15" s="8" t="str">
         <x:v>提示词包构建与下发：人设+提示词+作业策略 组装为提示词包(agent_id+版本)，经 II-14 同步 MC 持存</x:v>
       </x:c>
-      <x:c r="F15" t="str">
+      <x:c r="F15" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G15" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H15" t="str">
+      <x:c r="G15" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H15" s="8" t="str">
         <x:v>提示词人工填写，不是模型生成</x:v>
       </x:c>
-      <x:c r="I15" t="str">
+      <x:c r="I15" s="8" t="str">
         <x:v>MC agent-runtime 运行时依赖</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" t="str">
         <x:v>SWM-3</x:v>
       </x:c>
-      <x:c r="B16" t="str">
+      <x:c r="B16" s="8" t="str">
         <x:v>SWM</x:v>
       </x:c>
-      <x:c r="C16" t="str">
+      <x:c r="C16" s="8" t="str">
         <x:v>M-SWM-04</x:v>
       </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="D16" s="8" t="str">
         <x:v>R-SWM-002</x:v>
       </x:c>
-      <x:c r="E16" t="str">
+      <x:c r="E16" s="8" t="str">
         <x:v>蜂群记忆读写：swm-memory 服务提供记忆存取，被 MC agent-runtime 远程读取注入运行时</x:v>
       </x:c>
-      <x:c r="F16" t="str">
+      <x:c r="F16" s="13" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="G16" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H16" t="str">
+      <x:c r="G16" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H16" s="8" t="str">
         <x:v>记忆服务不可用→MC 无记忆降级运行</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17">
+      <x:c r="I16" s="8"/>
+    </x:row>
+    <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" t="str">
         <x:v>SWM-4</x:v>
       </x:c>
-      <x:c r="B17" t="str">
+      <x:c r="B17" s="8" t="str">
         <x:v>SWM</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C17" s="8" t="str">
         <x:v>M-SWM-02</x:v>
       </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="D17" s="8" t="str">
         <x:v>R-SWM-001</x:v>
       </x:c>
-      <x:c r="E17" t="str">
+      <x:c r="E17" s="8" t="str">
         <x:v>coze-loop Playground：魔改 coze-loop 接入，Web 试跑提示词看 IRS 输出(调 EI-05)</x:v>
       </x:c>
-      <x:c r="F17" t="str">
+      <x:c r="F17" s="15" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="G17" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H17" t="str">
+      <x:c r="G17" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H17" s="8" t="str">
         <x:v>魔改不成→砍 Playground，退 swm-gw 自研最简试运行</x:v>
       </x:c>
-      <x:c r="I17" t="str">
+      <x:c r="I17" s="8" t="str">
         <x:v>高风险项#2；演示多一个画面</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" t="str">
         <x:v>SWM-5</x:v>
       </x:c>
-      <x:c r="B18" t="str">
+      <x:c r="B18" s="8" t="str">
         <x:v>SWM</x:v>
       </x:c>
-      <x:c r="C18" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
+      <x:c r="C18" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E18" s="8" t="str">
         <x:v>（砍）评测集/评估器/实验(M-SWM-06)；自动生成提示词(M-SWM-07，依赖II-18 OCC画像)；swm-distill 提炼</x:v>
       </x:c>
       <x:c r="F18" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="G18" t="str">
+      <x:c r="G18" s="14" t="str">
         <x:v>砍</x:v>
       </x:c>
-      <x:c r="H18" t="str">
+      <x:c r="H18" s="8" t="str">
         <x:v>留 V1.1+</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19">
+      <x:c r="I18" s="8"/>
+    </x:row>
+    <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" t="str">
         <x:v>IRS-1</x:v>
       </x:c>
-      <x:c r="B19" t="str">
+      <x:c r="B19" s="8" t="str">
         <x:v>IRS</x:v>
       </x:c>
-      <x:c r="C19" t="str">
+      <x:c r="C19" s="8" t="str">
         <x:v>M-IRS-00</x:v>
       </x:c>
-      <x:c r="D19" t="str">
+      <x:c r="D19" s="8" t="str">
         <x:v>R-IRS-001</x:v>
       </x:c>
-      <x:c r="E19" t="str">
+      <x:c r="E19" s="8" t="str">
         <x:v>部署 1 个多模态视觉模型(如 Qwen2-VL/InternVL)；提供 EI-05 统一推理接口；私有化部署不依赖公有云</x:v>
       </x:c>
-      <x:c r="F19" t="str">
+      <x:c r="F19" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G19" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H19" t="str">
+      <x:c r="G19" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H19" s="8" t="str">
         <x:v>VLM效果差→智能体降级UI树+文本LLM；GPU不足→更小模型</x:v>
       </x:c>
-      <x:c r="I19" t="str">
+      <x:c r="I19" s="8" t="str">
         <x:v>高风险项#1；演示灵魂；CON-06私有化</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" t="str">
         <x:v>IRS-2</x:v>
       </x:c>
-      <x:c r="B20" t="str">
+      <x:c r="B20" s="8" t="str">
         <x:v>IRS</x:v>
       </x:c>
-      <x:c r="C20" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E20" t="str">
+      <x:c r="C20" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D20" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E20" s="8" t="str">
         <x:v>（砍）多模型管理/切换；完整推理监控；多租户配额</x:v>
       </x:c>
       <x:c r="F20" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="G20" t="str">
+      <x:c r="G20" s="14" t="str">
         <x:v>砍</x:v>
       </x:c>
-      <x:c r="H20" t="str">
+      <x:c r="H20" s="8" t="str">
         <x:v>固定单一模型</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21">
+      <x:c r="I20" s="8"/>
+    </x:row>
+    <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" t="str">
         <x:v>OCC-1</x:v>
       </x:c>
-      <x:c r="B21" t="str">
+      <x:c r="B21" s="8" t="str">
         <x:v>OCC</x:v>
       </x:c>
-      <x:c r="C21" t="str">
+      <x:c r="C21" s="8" t="str">
         <x:v>M-OCC-05</x:v>
       </x:c>
-      <x:c r="D21" t="str">
+      <x:c r="D21" s="8" t="str">
         <x:v>R-OCC-006</x:v>
       </x:c>
-      <x:c r="E21" t="str">
+      <x:c r="E21" s="8" t="str">
         <x:v>作战编排轻量版：Web 选一群智能体节点+任务节点 → 经 II-10 下发 MC 执行 → 效果数据回传</x:v>
       </x:c>
-      <x:c r="F21" t="str">
+      <x:c r="F21" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G21" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H21" t="str">
+      <x:c r="G21" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H21" s="8" t="str">
         <x:v>不做 Flowable/BPMN，用最简任务下发；不做中途改编排</x:v>
       </x:c>
-      <x:c r="I21" t="str">
+      <x:c r="I21" s="8" t="str">
         <x:v>蜂群唯一正宗驱动源</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" t="str">
         <x:v>OCC-2</x:v>
       </x:c>
-      <x:c r="B22" t="str">
+      <x:c r="B22" s="8" t="str">
         <x:v>OCC</x:v>
       </x:c>
-      <x:c r="C22" t="str">
+      <x:c r="C22" s="8" t="str">
         <x:v>M-OCC-01/06</x:v>
       </x:c>
-      <x:c r="D22" t="str">
+      <x:c r="D22" s="8" t="str">
         <x:v>R-OCC-001/007</x:v>
       </x:c>
-      <x:c r="E22" t="str">
+      <x:c r="E22" s="8" t="str">
         <x:v>预设数据看板：目标档案/作战效果用预设样本数据展示(Web 看板)，不做自动分析</x:v>
       </x:c>
-      <x:c r="F22" t="str">
+      <x:c r="F22" s="13" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="G22" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H22" t="str">
+      <x:c r="G22" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H22" s="8" t="str">
         <x:v>完全静态预设数据</x:v>
       </x:c>
-    </x:row>
-    <x:row r="23">
+      <x:c r="I22" s="8"/>
+    </x:row>
+    <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" t="str">
         <x:v>OCC-3</x:v>
       </x:c>
-      <x:c r="B23" t="str">
+      <x:c r="B23" s="8" t="str">
         <x:v>OCC</x:v>
       </x:c>
-      <x:c r="C23" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D23" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E23" t="str">
+      <x:c r="C23" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D23" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E23" s="8" t="str">
         <x:v>（砍）目标自动识别/分析研判(M-OCC-02)；效果评估模型(M-OCC-06)；策略库(M-OCC-07)；内容管理(M-OCC-08)；关系图谱</x:v>
       </x:c>
       <x:c r="F23" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="G23" t="str">
+      <x:c r="G23" s="14" t="str">
         <x:v>砍</x:v>
       </x:c>
-      <x:c r="H23" t="str">
+      <x:c r="H23" s="8" t="str">
         <x:v>留 V1.1+，相关环节人工</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24">
+      <x:c r="I23" s="8"/>
+    </x:row>
+    <x:row r="24" ht="48" customHeight="1">
       <x:c r="A24" t="str">
         <x:v>DC-1</x:v>
       </x:c>
-      <x:c r="B24" t="str">
+      <x:c r="B24" s="8" t="str">
         <x:v>DC</x:v>
       </x:c>
-      <x:c r="C24" t="str">
+      <x:c r="C24" s="8" t="str">
         <x:v>M-DC-02</x:v>
       </x:c>
-      <x:c r="D24" t="str">
+      <x:c r="D24" s="8" t="str">
         <x:v>R-DC-001</x:v>
       </x:c>
-      <x:c r="E24" t="str">
+      <x:c r="E24" s="8" t="str">
         <x:v>少量真采集：1-2 海外平台(如 X/TikTok)某话题帖子/用户数据进库，为 OCC 看板供原料</x:v>
       </x:c>
-      <x:c r="F24" t="str">
+      <x:c r="F24" s="15" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="G24" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H24" t="str">
+      <x:c r="G24" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H24" s="8" t="str">
         <x:v>采集不稳/被反爬→完全用预设样本数据替代</x:v>
       </x:c>
-      <x:c r="I24" t="str">
+      <x:c r="I24" s="8" t="str">
         <x:v>排期吃紧首个砍项(省Python栈)</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
+    <x:row r="25" ht="48" customHeight="1">
       <x:c r="A25" t="str">
         <x:v>DC-2</x:v>
       </x:c>
-      <x:c r="B25" t="str">
+      <x:c r="B25" s="8" t="str">
         <x:v>DC</x:v>
       </x:c>
-      <x:c r="C25" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D25" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E25" t="str">
+      <x:c r="C25" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D25" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E25" s="8" t="str">
         <x:v>（砍）代理池/调度限流/策略自优化；PySpark ETL；ClickHouse；情报回注闭环(M-DC-04)</x:v>
       </x:c>
       <x:c r="F25" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="G25" t="str">
+      <x:c r="G25" s="14" t="str">
         <x:v>砍</x:v>
       </x:c>
-      <x:c r="H25" t="str">
+      <x:c r="H25" s="8" t="str">
         <x:v>留 V1.1+</x:v>
       </x:c>
-    </x:row>
-    <x:row r="26">
+      <x:c r="I25" s="8"/>
+    </x:row>
+    <x:row r="26" ht="48" customHeight="1">
       <x:c r="A26" t="str">
         <x:v>COM-1</x:v>
       </x:c>
-      <x:c r="B26" t="str">
+      <x:c r="B26" s="8" t="str">
         <x:v>COM</x:v>
       </x:c>
-      <x:c r="C26" t="str">
+      <x:c r="C26" s="8" t="str">
         <x:v>M-COM-01</x:v>
       </x:c>
-      <x:c r="D26" t="str">
+      <x:c r="D26" s="8" t="str">
         <x:v>R-COM-001</x:v>
       </x:c>
-      <x:c r="E26" t="str">
+      <x:c r="E26" s="8" t="str">
         <x:v>登录+JWT签发；com-auth-lib 共享验签库(下沉每个Java服务本地验签)；1-2角色(管理员/操作员)；org_id 隔离</x:v>
       </x:c>
-      <x:c r="F26" t="str">
+      <x:c r="F26" s="13" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="G26" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H26" t="str">
+      <x:c r="G26" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H26" s="8" t="str">
         <x:v>com-auth-lib 可先简化为共享密钥本地校验</x:v>
       </x:c>
-      <x:c r="I26" t="str">
+      <x:c r="I26" s="8" t="str">
         <x:v>不做COM则各服务裸奔</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
+    <x:row r="27" ht="48" customHeight="1">
       <x:c r="A27" t="str">
         <x:v>COM-2</x:v>
       </x:c>
-      <x:c r="B27" t="str">
+      <x:c r="B27" s="8" t="str">
         <x:v>COM</x:v>
       </x:c>
-      <x:c r="C27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D27" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E27" t="str">
+      <x:c r="C27" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D27" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E27" s="8" t="str">
         <x:v>（砍）完整6角色×21权限RBAC；组织管理CRUD；5次锁定；令牌黑名单</x:v>
       </x:c>
       <x:c r="F27" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="G27" t="str">
+      <x:c r="G27" s="14" t="str">
         <x:v>砍</x:v>
       </x:c>
-      <x:c r="H27" t="str">
+      <x:c r="H27" s="8" t="str">
         <x:v>留 V1.1+</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28">
+      <x:c r="I27" s="8"/>
+    </x:row>
+    <x:row r="28" ht="48" customHeight="1">
       <x:c r="A28" t="str">
         <x:v>OM-1</x:v>
       </x:c>
-      <x:c r="B28" t="str">
+      <x:c r="B28" s="8" t="str">
         <x:v>OM</x:v>
       </x:c>
-      <x:c r="C28" t="str">
+      <x:c r="C28" s="8" t="str">
         <x:v>M-OM-01</x:v>
       </x:c>
-      <x:c r="D28" t="str">
+      <x:c r="D28" s="8" t="str">
         <x:v>R-OM-001</x:v>
       </x:c>
-      <x:c r="E28" t="str">
+      <x:c r="E28" s="8" t="str">
         <x:v>最小日志/任务看板：各子系统上报的关键日志、设备在线状态、任务执行状态 Web 可见</x:v>
       </x:c>
-      <x:c r="F28" t="str">
+      <x:c r="F28" s="15" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="G28" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H28" t="str">
+      <x:c r="G28" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H28" s="8" t="str">
         <x:v>只做关键日志聚合，不做指标检索/告警</x:v>
       </x:c>
-    </x:row>
-    <x:row r="29">
+      <x:c r="I28" s="8"/>
+    </x:row>
+    <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" t="str">
         <x:v>OM-2</x:v>
       </x:c>
-      <x:c r="B29" t="str">
+      <x:c r="B29" s="8" t="str">
         <x:v>OM</x:v>
       </x:c>
-      <x:c r="C29" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D29" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E29" t="str">
+      <x:c r="C29" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D29" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E29" s="8" t="str">
         <x:v>（砍）KubeSphere底座；Prometheus/Grafana；Alertmanager告警；OpenSearch日志检索</x:v>
       </x:c>
       <x:c r="F29" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="G29" t="str">
+      <x:c r="G29" s="14" t="str">
         <x:v>砍</x:v>
       </x:c>
-      <x:c r="H29" t="str">
+      <x:c r="H29" s="8" t="str">
         <x:v>留 V1.1+</x:v>
       </x:c>
-    </x:row>
-    <x:row r="30">
+      <x:c r="I29" s="8"/>
+    </x:row>
+    <x:row r="30" ht="48" customHeight="1">
       <x:c r="A30" t="str">
         <x:v>FE-1</x:v>
       </x:c>
-      <x:c r="B30" t="str">
+      <x:c r="B30" s="8" t="str">
         <x:v>前端</x:v>
       </x:c>
-      <x:c r="C30" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D30" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E30" t="str">
+      <x:c r="C30" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D30" s="8" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E30" s="8" t="str">
         <x:v>Web 控制台：登录页/控制台门户/MC终端台账/远程控制页(单控+宫格)/OCC编排页/SWM提示词页/OM看板</x:v>
       </x:c>
-      <x:c r="F30" t="str">
+      <x:c r="F30" s="11" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G30" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="H30" t="str">
+      <x:c r="G30" s="12" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="H30" s="8" t="str">
         <x:v>参考线框稿(.pen)已有 63 页设计，MVP 实现~10 核心页</x:v>
       </x:c>
-      <x:c r="I30" t="str">
+      <x:c r="I30" s="8" t="str">
         <x:v>Vue3/React+TS</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:pageSetup fitToWidth="1" fitToHeight="0" orientation="landscape"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF548235"/>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
+  <x:cols>
+    <x:col min="1" max="1" width="18" customWidth="1"/>
+    <x:col min="2" max="2" width="12" customWidth="1"/>
+    <x:col min="3" max="3" width="20" customWidth="1"/>
+    <x:col min="4" max="4" width="62" customWidth="1"/>
+    <x:col min="5" max="5" width="40" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>MVP 阶段排期（3 个月 · 2-4 人）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="9" t="str">
+        <x:v>阶段按演示主线倒推：先打通 MC 执行链路 + IRS 多模态（演示灵魂），再补 SWM/OCC 驱动源，最后 OCC/DC 闭环 + 联调演示。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="7" t="str">
+        <x:v>阶段</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="str">
+        <x:v>时间窗</x:v>
+      </x:c>
+      <x:c r="C4" s="7" t="str">
+        <x:v>里程碑</x:v>
+      </x:c>
+      <x:c r="D4" s="7" t="str">
+        <x:v>主要工作</x:v>
+      </x:c>
+      <x:c r="E4" s="7" t="str">
+        <x:v>交付物</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="72" customHeight="1">
+      <x:c r="A5" t="str">
+        <x:v>第0阶段·地基</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>第1-2周</x:v>
+      </x:c>
+      <x:c r="C5" s="8" t="str">
+        <x:v>M0：能登录</x:v>
+      </x:c>
+      <x:c r="D5" s="8" t="str">
+        <x:v>COM 登录+JWT+com-auth-lib(各Java服务接入)；开发环境搭建(K8s/PG/Redis/MinIO)；前端骨架(登录/门户)；MC 真机ADB接入打通1台</x:v>
+      </x:c>
+      <x:c r="E5" s="8" t="str">
+        <x:v>可登录的控制台骨架 + 1台真机ADB可见</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="72" customHeight="1">
+      <x:c r="A6" t="str">
+        <x:v>第1阶段·演示灵魂</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>第3-6周</x:v>
+      </x:c>
+      <x:c r="C6" s="16" t="str">
+        <x:v>M1：智能体能动★</x:v>
+      </x:c>
+      <x:c r="D6" s="8" t="str">
+        <x:v>IRS 部署多模态模型+EI-05接口；MC 执行网关收口；agent-runtime 调IRS视觉推理→动作→经网关落地；mc-sfu 单控WebRTC+宫格；脚本引擎GraalVM。★早期验证点：截图→推理→动作能跑通一次</x:v>
+      </x:c>
+      <x:c r="E6" s="8" t="str">
+        <x:v>单台真机：智能体看屏幕自主决策 + WebRTC远控画面</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="72" customHeight="1">
+      <x:c r="A7" t="str">
+        <x:v>第2阶段·提示词供给</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>第7-9周</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>M2：提示词能驱动</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>SWM swm-gw/swm-memory；人设录入+提示词包构建；II-14同步MC持存；记忆读写；coze-loop Playground(魔改，时间盒3周，不成则砍退自研简版)；多台真机(扩到3-8台)宫格同时跑</x:v>
+      </x:c>
+      <x:c r="E7" s="8" t="str">
+        <x:v>一群智能体按各自人设+提示词包在多台真机上作业</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" customHeight="1">
+      <x:c r="A8" t="str">
+        <x:v>第3阶段·闭环驱动</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>第10-11周</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>M3：蜂群能编排</x:v>
+      </x:c>
+      <x:c r="D8" s="8" t="str">
+        <x:v>OCC 作战编排轻量版：Web选智能体群+任务→II-10下发MC→效果回传；OCC预设数据看板；DC少量真采集供料(不稳则退预设数据)；OM最小日志看板</x:v>
+      </x:c>
+      <x:c r="E8" s="8" t="str">
+        <x:v>OCC编排驱动蜂群执行 + 效果看板</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="72" customHeight="1">
+      <x:c r="A9" t="str">
+        <x:v>第4阶段·联调演示</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>第12-13周</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>M4：可演示</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="str">
+        <x:v>全链路联调(登录→SWM提示词→OCC编排→MC执行→IRS推理→效果回传→OM看板)；演示脚本打磨；稳定性收尾；写说明文档</x:v>
+      </x:c>
+      <x:c r="E9" s="8" t="str">
+        <x:v>可现场演示的完整系统 + 说明文档</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageSetup fitToWidth="1" fitToHeight="1" orientation="landscape"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFC00000"/>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
+  <x:cols>
+    <x:col min="1" max="1" width="6" customWidth="1"/>
+    <x:col min="2" max="2" width="42" customWidth="1"/>
+    <x:col min="3" max="3" width="6" customWidth="1"/>
+    <x:col min="4" max="4" width="42" customWidth="1"/>
+    <x:col min="5" max="5" width="50" customWidth="1"/>
+    <x:col min="6" max="6" width="30" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>MVP 风险登记</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="7" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="str">
+        <x:v>风险项</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="str">
+        <x:v>等级</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="str">
+        <x:v>影响</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="str">
+        <x:v>应对/降级路径</x:v>
+      </x:c>
+      <x:c r="F3" s="7" t="str">
+        <x:v>触发判断点</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="66" customHeight="1">
+      <x:c r="A4" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="B4" s="8" t="str">
+        <x:v>多模态视觉模型驱动手机 GUI 效果差/延迟高（演示灵魂，不探针直接赌）</x:v>
+      </x:c>
+      <x:c r="C4" s="17" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>演示主线（智能体看屏幕自主决策）崩塌，脚本兜底救不了『智能体』主语，整个 MVP 定位失败</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>降级 UI树(a11y dump)+纯文本LLM推理（不看图但仍是智能体）；GPU不足用更小参数模型；演示选 VLM 表现好的场景</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>第4-6周早期验证点：截图→推理→动作能否跑通一次。跑不通即触发降级</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="66" customHeight="1">
+      <x:c r="A5" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="B5" s="8" t="str">
+        <x:v>coze-loop 魔改不成（硬投入，SWM Playground 依赖）</x:v>
+      </x:c>
+      <x:c r="C5" s="18" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="D5" s="8" t="str">
+        <x:v>SWM 演示少一个『提示词调优』画面，但不影响主链路（演示灵魂在 MC/IRS）</x:v>
+      </x:c>
+      <x:c r="E5" s="8" t="str">
+        <x:v>硬止损：时间盒3周，魔改不成→砍 Playground，退 swm-gw 自研最简试运行(输入提示词→调IRS→看输出)</x:v>
+      </x:c>
+      <x:c r="F5" s="8" t="str">
+        <x:v>第7-9周末：coze-loop 能否调通试跑</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="66" customHeight="1">
+      <x:c r="A6" t="str">
+        <x:v>R3</x:v>
+      </x:c>
+      <x:c r="B6" s="8" t="str">
+        <x:v>mc-sfu 自建 mediasoup WebRTC 联调复杂（真机画面回传）</x:v>
+      </x:c>
+      <x:c r="C6" s="18" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="D6" s="8" t="str">
+        <x:v>远控画面不可用，宫格『一片设备同时在动』的视觉冲击减弱</x:v>
+      </x:c>
+      <x:c r="E6" s="8" t="str">
+        <x:v>mc-sfu 故障降级截图轮询；宫格先做截图刷新</x:v>
+      </x:c>
+      <x:c r="F6" s="8" t="str">
+        <x:v>第3-6周：WebRTC 单控能否出画面</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="66" customHeight="1">
+      <x:c r="A7" t="str">
+        <x:v>R4</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>范围 vs 时间：5子系统5技术栈在3月2-4人下满负荷偏紧</x:v>
+      </x:c>
+      <x:c r="C7" s="18" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>后期质量塌方或延期</x:v>
+      </x:c>
+      <x:c r="E7" s="8" t="str">
+        <x:v>排期吃紧按优先级砍：先砍 DC 真采集(退预设数据，省Python栈)→再砍 coze-loop Playground→再砍 OM/COM 非核心；绝不砍 MC执行链路+IRS多模态</x:v>
+      </x:c>
+      <x:c r="F7" s="8" t="str">
+        <x:v>每个里程碑评审是否达标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="66" customHeight="1">
+      <x:c r="A8" t="str">
+        <x:v>R5</x:v>
+      </x:c>
+      <x:c r="B8" s="8" t="str">
+        <x:v>真机账号被平台风控/封禁（真实账号在真实平台作业）</x:v>
+      </x:c>
+      <x:c r="C8" s="18" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="D8" s="8" t="str">
+        <x:v>演示账号失效，无法演示</x:v>
+      </x:c>
+      <x:c r="E8" s="8" t="str">
+        <x:v>备用账号池；演示用养好的账号；脚本模式拟人化节奏(M-MC-09)</x:v>
+      </x:c>
+      <x:c r="F8" s="8" t="str">
+        <x:v>演示前账号健康检查</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageSetup fitToWidth="1" fitToHeight="1" orientation="landscape"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-07-20 17:46:04
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/MVP功能清单.xlsx
+++ b/公司项目/认知作战/文档/MVP功能清单.xlsx
@@ -1521,7 +1521,7 @@
           <x:t>编制日期</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" s="61">
+      <x:c r="B7" s="77" t="n">
         <x:v>46223</x:v>
       </x:c>
     </x:row>
@@ -1537,10 +1537,11 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="55" customHeight="1">
-      <x:c r="A10" s="3" t="str">
-        <x:v>本清单是「认知行动平台」全量功能（7 子系统 40 项需求下的全部模块/功能点）的分版本交付规划。基于《MVP 版本规划》与线框图（认知作战平台-线框图.pen，37 业务页+5 横切页），将全部功能分 4 档版本（V1.0~V1.3）落地，明确每项功能：所属版本、优先级、类型(前端页/后端模块/全栈)、依赖项、工期(人天)、完成人、对应页面·模块。</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="str"/>
+      <x:c r="A10" s="3" t="inlineStr">
+        <x:is>
+          <x:t>本清单是「认知行动平台」全量功能（7 子系统 40 项需求下的全部模块/功能点）的分版本交付规划。基于《MVP 版本规划》与线框图（认知作战平台-线框图.pen，37 业务页+5 横切页），将全部功能分 4 档版本（V1.0~V1.3）落地，明确每项功能：所属版本、优先级、类型(前端页/后端模块/全栈)、依赖项、工期(人天)、完成人、对应页面·模块。</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="46" t="inlineStr">
@@ -1551,9 +1552,8 @@
     </x:row>
     <x:row r="12" ht="55" customHeight="1">
       <x:c r="A12" s="63" t="str">
-        <x:v>V1.0=可演示最小闭环（演示主链路，第1-4月，22页+后端执行链）；V1.1=线框图补齐（第5-7月，15页+评测/系统管理）；V1.2=后台增强（第8-10月，桌面端/指标告警/调度/情报分析）；V1.3=深化（第11-12月，IRS多模型/OCC策略库内容图谱Flowable/完整RBAC）。共 12 月 · 6 人（后端5+前端1）。</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="str"/>
+        <x:v>V1.0=可演示最小闭环+系统管理控制台（演示主链路+COM若依11页，第1-4月，33页+后端执行链）；V1.1=线框图补齐（第5-7月，10页：MC 6+OCC评估1+SWM评测3）；V1.2=后台增强（第8-10月，桌面端/指标告警/调度/情报分析）；V1.3=深化（第11-12月，IRS多模型/OCC策略库内容图谱Flowable/完整RBAC）。共 12 月 · 6 人（后端5+前端1）。</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="46" t="inlineStr">
@@ -1563,10 +1563,11 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="55" customHeight="1">
-      <x:c r="A14" s="3" t="str">
-        <x:v>后1=MC执行链(M-MC-01/03/04/05/06)；后2=MC业务链(M-MC-07/08/10/11/14)；后3=SWM+IRS(M-SWM+M-IRS+coze-loop Go)；后4=OCC(M-OCC全)；后5=COM+DC+OM(M-COM+M-DC+M-OM)；前1=前端(Vue3，4控制台+5横切页，42业务页全做)。</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="str"/>
+      <x:c r="A14" s="3" t="inlineStr">
+        <x:is>
+          <x:t>后1=MC执行链(M-MC-01/03/04/05/06)；后2=MC业务链(M-MC-07/08/10/11/14)；后3=SWM+IRS(M-SWM+M-IRS+coze-loop Go)；后4=OCC(M-OCC全)；后5=COM+DC+OM(M-COM+M-DC+M-OM)；前1=前端(Vue3，4控制台+5横切页，42业务页全做)。</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="62" t="inlineStr">
@@ -1576,10 +1577,11 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="55" customHeight="1">
-      <x:c r="A16" s="3" t="str">
-        <x:v>CON-07 动作收口：所有真机动作经 MC 执行网关落地（可观测/可审计/可熔断）；CON-10 推理与执行分离：agent-runtime 调 IRS 视觉推理不经网关，产出的动作指令再经网关落地；CON-08 双执行模式：脚本模式保底（确定性流程）+ 智能体模式亮点（VLM 视觉决策）。</x:v>
-      </x:c>
-      <x:c r="B16" s="3" t="str"/>
+      <x:c r="A16" s="3" t="inlineStr">
+        <x:is>
+          <x:t>CON-07 动作收口：所有真机动作经 MC 执行网关落地（可观测/可审计/可熔断）；CON-10 推理与执行分离：agent-runtime 调 IRS 视觉推理不经网关，产出的动作指令再经网关落地；CON-08 双执行模式：脚本模式保底（确定性流程）+ 智能体模式亮点（VLM 视觉决策）。</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="46" t="inlineStr">
@@ -1589,10 +1591,11 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
-      <x:c r="A18" s="63" t="str">
-        <x:v>P0=必做（演示灵魂/架构底线）；P1=应做（核心支撑）；P2=可缓（配角/锦上添花，按版本里程碑弹性调整）。</x:v>
-      </x:c>
-      <x:c r="B18" s="3" t="str"/>
+      <x:c r="A18" s="63" t="inlineStr">
+        <x:is>
+          <x:t>P0=必做（演示灵魂/架构底线）；P1=应做（核心支撑）；P2=可缓（配角/锦上添花，按版本里程碑弹性调整）。</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="46" t="inlineStr">
@@ -1602,10 +1605,11 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
-      <x:c r="A20" s="3" t="str">
-        <x:v>前端页=纯前端页面（前1完成）；后端模块=纯后端模块（后1~后5完成）；全栈=前后端都涉及（如 后1+前1）。</x:v>
-      </x:c>
-      <x:c r="B20" s="3" t="str"/>
+      <x:c r="A20" s="3" t="inlineStr">
+        <x:is>
+          <x:t>前端页=纯前端页面（前1完成）；后端模块=纯后端模块（后1~后5完成）；全栈=前后端都涉及（如 后1+前1）。</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="62" t="inlineStr">
@@ -1615,10 +1619,11 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="40" customHeight="1">
-      <x:c r="A22" s="60" t="str">
-        <x:v>人天（per人·天）。1人周=5人天（按工作日）。如 10人天=1人做10天 或 2人做5天。模块行(②模块)不单独给工期，工期汇总其下功能行。</x:v>
-      </x:c>
-      <x:c r="B22" s="60" t="str"/>
+      <x:c r="A22" s="60" t="inlineStr">
+        <x:is>
+          <x:t>人天（per人·天）。1人周=5人天（按工作日）。如 10人天=1人做10天 或 2人做5天。模块行(②模块)不单独给工期，工期汇总其下功能行。</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C22" s="29" t="n"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
@@ -1768,22 +1773,22 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells count="16">
+    <x:mergeCell ref="A20:B20"/>
     <x:mergeCell ref="A21:B21"/>
+    <x:mergeCell ref="A16:B16"/>
     <x:mergeCell ref="A15:B15"/>
     <x:mergeCell ref="A19:B19"/>
     <x:mergeCell ref="A11:B11"/>
+    <x:mergeCell ref="A10:B10"/>
     <x:mergeCell ref="A13:B13"/>
+    <x:mergeCell ref="A14:B14"/>
     <x:mergeCell ref="A1:B1"/>
     <x:mergeCell ref="A23:B23"/>
     <x:mergeCell ref="A9:B9"/>
     <x:mergeCell ref="A17:B17"/>
-    <x:mergeCell ref="A10:B10"/>
+    <x:mergeCell ref="A18:B18"/>
+    <x:mergeCell ref="A22:B22"/>
     <x:mergeCell ref="A12:B12"/>
-    <x:mergeCell ref="A14:B14"/>
-    <x:mergeCell ref="A16:B16"/>
-    <x:mergeCell ref="A18:B18"/>
-    <x:mergeCell ref="A20:B20"/>
-    <x:mergeCell ref="A22:B22"/>
   </x:mergeCells>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <x:pageSetup paperSize="1" orientation="landscape"/>
@@ -1870,20 +1875,14 @@
           <x:t>M0：能登录</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="53" t="inlineStr">
-        <x:is>
-          <x:t>COM登录+JWT+com-auth-lib(各Java服务接入)；开发环境搭建(K8s/PG/Redis/MinIO)；前端骨架(登录/门户)；MC真机ADB接入打通1台</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="53" t="inlineStr">
-        <x:is>
-          <x:t>后5(COM)+前1(骨架)；后1(MC ADB打通)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F4" s="54" t="inlineStr">
-        <x:is>
-          <x:t>可登录的控制台骨架 + 1台真机ADB可见</x:t>
-        </x:is>
+      <x:c r="D4" s="53" t="str">
+        <x:v>COM若依原生登录(/login+/getInfo+/getRouters)+Token签发+Redis共享校验+跨控制台SSO；系统管理控制台11页(若依原生：用户/角色/部门/登录策略/登录日志/菜单/岗位/字典/参数/通知/操作日志)+部门成员管理；开发环境搭建(K8s/PG/Redis/MinIO)；前端骨架(登录/门户)；MC真机ADB接入打通1台</x:v>
+      </x:c>
+      <x:c r="E4" s="53" t="str">
+        <x:v>后5(COM登录+系统管理11页)+前1(骨架+11页)；后1(MC ADB打通)</x:v>
+      </x:c>
+      <x:c r="F4" s="54" t="str">
+        <x:v>可登录的控制台骨架 + 系统管理控制台11页 + 1台真机ADB可见</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="90" customHeight="1">
@@ -1998,20 +1997,14 @@
           <x:t>M4：线框图补齐</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="56" t="inlineStr">
-        <x:is>
-          <x:t>MC补6页(分组/代理池/模板/编排器/IDE/审计)；OCC-13评估；SWM评测3页(评测集/评估器/实验)；系统管理控制台(若依风格11页)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E8" s="56" t="inlineStr">
-        <x:is>
-          <x:t>后1(MC编排/IDE)+后2(MC审计)+后3(SWM评测)+后4(OCC评估)+后5(COM系统管理)+前1(15页)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F8" s="56" t="inlineStr">
-        <x:is>
-          <x:t>线框图全 37 业务页 + 5 横切页落地</x:t>
-        </x:is>
+      <x:c r="D8" s="56" t="str">
+        <x:v>MC补6页(分组/代理池/模板/编排器/IDE/审计)；OCC-13评估；SWM评测3页(评测集/评估器/实验)</x:v>
+      </x:c>
+      <x:c r="E8" s="56" t="str">
+        <x:v>后1(MC编排/IDE)+后2(MC审计)+后3(SWM评测)+后4(OCC评估)+前1(4页)</x:v>
+      </x:c>
+      <x:c r="F8" s="56" t="str">
+        <x:v>线框图剩余业务页落地（MC 6 + OCC 1 + SWM 3 = 10页）</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="90" customHeight="1">
@@ -2627,22 +2620,18 @@
       </x:c>
       <x:c r="D9" s="36" t="inlineStr">
         <x:is>
-          <x:t>Java(Spring Boot：com-service)+Spring Security+JJWT+PostgreSQL+Redis</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" s="36" t="inlineStr">
-        <x:is>
-          <x:t>登录+JWT签发；com-auth-lib共享验签库；1-2角色(管理员/操作员)；org_id隔离。5横切页(G-01~05)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F9" s="36" t="inlineStr">
-        <x:is>
-          <x:t>系统管理控制台(若依风格11页)：用户/角色/部门/登录策略/登录日志/菜单/岗位/字典/参数/通知/操作日志；组织成员管理</x:t>
-        </x:is>
+          <x:t>Java(Spring Boot：com-service 基于若依)+若依原生认证+Redis共享校验+PostgreSQL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="36" t="str">
+        <x:v>若依原生登录(/login+/getInfo+/getRouters)；有状态Token(uuid+Base64存Redis)；各子系统查共享Redis校验；跨4控制台SSO；1-2角色(sys_role)；部门数据权限(@DataScope)；5横切页(G-01~05)；系统管理控制台11页(若依原生：用户/角色/部门/登录策略/登录日志/菜单/岗位/字典/参数/通知/操作日志)+部门成员管理</x:v>
+      </x:c>
+      <x:c r="F9" s="36" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="G9" s="36" t="inlineStr">
         <x:is>
-          <x:t>完整6角色×21权限RBAC；5次锁定策略；令牌黑名单/登出吊毁</x:t>
+          <x:t>若依完整RBAC：多角色+细粒度菜单/按钮权限点+@PreAuthorize+@DataScope全套；5次锁定策略；令牌黑名单/登出吊毁</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -10034,10 +10023,8 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
-      <x:c r="A4" s="9" t="inlineStr">
-        <x:is>
-          <x:t>【V1.0 · 登录底座】（第 1-4 月 · 后5+前1）</x:t>
-        </x:is>
+      <x:c r="A4" s="9" t="str">
+        <x:v>【V1.0 · 登录底座 + 系统管理控制台】（第 1-4 月 · 后5+前1）</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
@@ -10068,7 +10055,7 @@
       </x:c>
       <x:c r="F5" s="35" t="inlineStr">
         <x:is>
-          <x:t>登录+JWT签发</x:t>
+          <x:t>若依原生登录+Token签发+Redis共享校验+跨控制台SSO</x:t>
         </x:is>
       </x:c>
       <x:c r="G5" s="35" t="inlineStr">
@@ -10131,7 +10118,7 @@
       </x:c>
       <x:c r="F6" s="78" t="inlineStr">
         <x:is>
-          <x:t>登录+JWT签发</x:t>
+          <x:t>若依原生登录（/login 校验+签发 /getInfo 取用户信息 /getRouters 取动态菜单）</x:t>
         </x:is>
       </x:c>
       <x:c r="G6" s="78" t="inlineStr">
@@ -10164,7 +10151,7 @@
       </x:c>
       <x:c r="M6" s="36" t="str"/>
     </x:row>
-    <x:row r="7" ht="40" customHeight="1">
+    <x:row r="7" ht="55" customHeight="1">
       <x:c r="A7" s="36" t="inlineStr">
         <x:is>
           <x:t>③功能</x:t>
@@ -10177,7 +10164,7 @@
       </x:c>
       <x:c r="C7" s="36" t="inlineStr">
         <x:is>
-          <x:t>认证令牌签发</x:t>
+          <x:t>令牌签发与 Redis 共享校验</x:t>
         </x:is>
       </x:c>
       <x:c r="D7" s="36" t="inlineStr">
@@ -10192,7 +10179,7 @@
       </x:c>
       <x:c r="F7" s="78" t="inlineStr">
         <x:is>
-          <x:t>JWT签发+com-auth-lib本地验签</x:t>
+          <x:t>若依有状态 Token 签发（uuid + Base64 用户信息存 Redis login_tokens:{uuid}）；各子系统查共享 Redis 校验，无 com-auth-lib</x:t>
         </x:is>
       </x:c>
       <x:c r="G7" s="78" t="inlineStr">
@@ -10225,264 +10212,326 @@
       </x:c>
       <x:c r="M7" s="36" t="inlineStr">
         <x:is>
-          <x:t>可简化共享密钥</x:t>
+          <x:t>基于若依原生；废弃JWT+com-auth-lib；共享Redis校验</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="8" ht="40" customHeight="1">
-      <x:c r="A8" s="79" t="inlineStr">
+      <x:c r="A8" s="36" t="inlineStr">
         <x:is>
           <x:t>③功能</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="79" t="inlineStr">
+      <x:c r="B8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>F-COM-01-04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>跨控制台 SSO 会话</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>R-COM-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>V1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="78" t="inlineStr">
+        <x:is>
+          <x:t>令牌跨 4 控制台（MC/OCC/SWM/系统管理）共享，一次登录通用；前端令牌存 localStorage，跳转控制台免登</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="78" t="inlineStr">
+        <x:is>
+          <x:t>P1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>全栈</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>F-COM-01-03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J8" s="36" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>后5+前1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>G-01~G-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M8" s="36" t="inlineStr">
+        <x:is>
+          <x:t>SSO核心；共享Redis+前端令牌传递</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="40" customHeight="1">
+      <x:c r="A9" s="79" t="inlineStr">
+        <x:is>
+          <x:t>③功能</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="79" t="inlineStr">
         <x:is>
           <x:t>G-01~05页</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="79" t="inlineStr">
+      <x:c r="C9" s="79" t="inlineStr">
         <x:is>
           <x:t>SSO横切页（登录/门户/个人中心/错误/通知）</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="79" t="inlineStr">
+      <x:c r="D9" s="79" t="inlineStr">
         <x:is>
           <x:t>R-COM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" s="79" t="inlineStr">
+      <x:c r="E9" s="79" t="inlineStr">
         <x:is>
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F8" s="80" t="inlineStr">
+      <x:c r="F9" s="80" t="inlineStr">
         <x:is>
           <x:t>5个横切通用页</x:t>
         </x:is>
       </x:c>
-      <x:c r="G8" s="80" t="inlineStr">
+      <x:c r="G9" s="80" t="inlineStr">
         <x:is>
           <x:t>P1</x:t>
         </x:is>
       </x:c>
-      <x:c r="H8" s="79" t="inlineStr">
+      <x:c r="H9" s="79" t="inlineStr">
         <x:is>
           <x:t>前端页</x:t>
         </x:is>
       </x:c>
-      <x:c r="I8" s="79" t="inlineStr">
+      <x:c r="I9" s="79" t="inlineStr">
         <x:is>
           <x:t>F-COM-01-01</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" s="36" t="n">
+      <x:c r="J9" s="36" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K8" s="36" t="inlineStr">
+      <x:c r="K9" s="36" t="inlineStr">
         <x:is>
           <x:t>前1</x:t>
         </x:is>
       </x:c>
-      <x:c r="L8" s="36" t="inlineStr">
+      <x:c r="L9" s="36" t="inlineStr">
         <x:is>
           <x:t>G-01~G-05</x:t>
         </x:is>
       </x:c>
-      <x:c r="M8" s="36" t="inlineStr">
+      <x:c r="M9" s="36" t="inlineStr">
         <x:is>
           <x:t>M-COM-01/02</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="40" customHeight="1">
-      <x:c r="A9" s="10" t="inlineStr">
+    <x:row r="10" ht="40" customHeight="1">
+      <x:c r="A10" s="10" t="inlineStr">
         <x:is>
           <x:t>②模块</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="10" t="inlineStr">
+      <x:c r="B10" s="10" t="inlineStr">
         <x:is>
           <x:t>M-COM-02</x:t>
         </x:is>
       </x:c>
-      <x:c r="C9" s="10" t="inlineStr">
+      <x:c r="C10" s="10" t="inlineStr">
         <x:is>
           <x:t>权限与组织管理</x:t>
         </x:is>
       </x:c>
-      <x:c r="D9" s="10" t="inlineStr">
+      <x:c r="D10" s="10" t="inlineStr">
         <x:is>
           <x:t>R-COM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="E9" s="10" t="inlineStr">
+      <x:c r="E10" s="10" t="inlineStr">
         <x:is>
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F9" s="35" t="inlineStr">
-        <x:is>
-          <x:t>1-2角色+org_id隔离</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G9" s="35" t="inlineStr">
-        <x:is>
-          <x:t>—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H9" s="10" t="inlineStr">
+      <x:c r="F10" s="35" t="inlineStr">
+        <x:is>
+          <x:t>若依原生角色权限(sys_role)+部门数据权限(@DataScope dept_id)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="35" t="inlineStr">
+        <x:is>
+          <x:t>—</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" s="10" t="inlineStr">
         <x:is>
           <x:t>后端模块</x:t>
         </x:is>
       </x:c>
-      <x:c r="I9" s="10" t="inlineStr">
+      <x:c r="I10" s="10" t="inlineStr">
         <x:is>
           <x:t>F-COM-01-01</x:t>
         </x:is>
       </x:c>
-      <x:c r="J9" s="10" t="inlineStr">
-        <x:is>
-          <x:t>—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K9" s="10" t="inlineStr">
-        <x:is>
-          <x:t>—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L9" s="10" t="str"/>
-      <x:c r="M9" s="10" t="str"/>
-    </x:row>
-    <x:row r="10" ht="40" customHeight="1">
-      <x:c r="A10" s="36" t="inlineStr">
+      <x:c r="J10" s="10" t="inlineStr">
+        <x:is>
+          <x:t>—</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K10" s="10" t="inlineStr">
+        <x:is>
+          <x:t>—</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L10" s="10" t="str"/>
+      <x:c r="M10" s="10" t="str"/>
+    </x:row>
+    <x:row r="11" ht="40" customHeight="1">
+      <x:c r="A11" s="36" t="inlineStr">
         <x:is>
           <x:t>③功能</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="36" t="inlineStr">
+      <x:c r="B11" s="36" t="inlineStr">
         <x:is>
           <x:t>F-COM-02-01</x:t>
         </x:is>
       </x:c>
-      <x:c r="C10" s="36" t="inlineStr">
+      <x:c r="C11" s="36" t="inlineStr">
         <x:is>
           <x:t>RBAC权限决策</x:t>
         </x:is>
       </x:c>
-      <x:c r="D10" s="36" t="inlineStr">
+      <x:c r="D11" s="36" t="inlineStr">
         <x:is>
           <x:t>R-COM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="E10" s="36" t="inlineStr">
+      <x:c r="E11" s="36" t="inlineStr">
         <x:is>
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F10" s="78" t="inlineStr">
-        <x:is>
-          <x:t>1-2角色(管理员/操作员)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G10" s="78" t="inlineStr">
+      <x:c r="F11" s="78" t="inlineStr">
+        <x:is>
+          <x:t>若依原生角色权限（sys_role + sys_role_menu + role_key）；1-2角色(管理员/操作员)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="78" t="inlineStr">
         <x:is>
           <x:t>P2</x:t>
         </x:is>
       </x:c>
-      <x:c r="H10" s="36" t="inlineStr">
+      <x:c r="H11" s="36" t="inlineStr">
         <x:is>
           <x:t>后端模块</x:t>
         </x:is>
       </x:c>
-      <x:c r="I10" s="36" t="inlineStr">
+      <x:c r="I11" s="36" t="inlineStr">
         <x:is>
           <x:t>F-COM-01-01</x:t>
         </x:is>
       </x:c>
-      <x:c r="J10" s="36" t="n">
+      <x:c r="J11" s="36" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="K10" s="36" t="inlineStr">
+      <x:c r="K11" s="36" t="inlineStr">
         <x:is>
           <x:t>后5</x:t>
         </x:is>
       </x:c>
-      <x:c r="L10" s="36" t="inlineStr">
-        <x:is>
-          <x:t>—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M10" s="36" t="inlineStr">
-        <x:is>
-          <x:t>不做完整RBAC</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15.75" customHeight="1">
-      <x:c r="A11" s="79" t="inlineStr">
+      <x:c r="L11" s="36" t="inlineStr">
+        <x:is>
+          <x:t>—</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M11" s="36" t="inlineStr">
+        <x:is>
+          <x:t>基于若依sys_role；不做完整RBAC</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="45" customHeight="1">
+      <x:c r="A12" s="79" t="inlineStr">
         <x:is>
           <x:t>③功能</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="36" t="inlineStr">
+      <x:c r="B12" s="36" t="inlineStr">
         <x:is>
           <x:t>F-COM-02-03</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" s="36" t="inlineStr">
-        <x:is>
-          <x:t>多组织数据隔离</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" s="36" t="inlineStr">
+      <x:c r="C12" s="36" t="inlineStr">
+        <x:is>
+          <x:t>部门数据权限（若依原生）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="36" t="inlineStr">
         <x:is>
           <x:t>R-COM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="E11" s="36" t="inlineStr">
+      <x:c r="E12" s="36" t="inlineStr">
         <x:is>
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F11" s="36" t="inlineStr">
-        <x:is>
-          <x:t>org_id行级隔离</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G11" s="36" t="inlineStr">
+      <x:c r="F12" s="36" t="inlineStr">
+        <x:is>
+          <x:t>若依原生 @DataScope 注解 + dept_id 数据权限（全部/本部门/本部门及以下/仅本人）；替代原 org_id 多组织隔离</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="36" t="inlineStr">
         <x:is>
           <x:t>P2</x:t>
         </x:is>
       </x:c>
-      <x:c r="H11" s="36" t="inlineStr">
+      <x:c r="H12" s="36" t="inlineStr">
         <x:is>
           <x:t>后端模块</x:t>
         </x:is>
       </x:c>
-      <x:c r="I11" s="36" t="inlineStr">
+      <x:c r="I12" s="36" t="inlineStr">
         <x:is>
           <x:t>F-COM-02-01</x:t>
         </x:is>
       </x:c>
-      <x:c r="J11" s="36" t="n">
+      <x:c r="J12" s="36" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K11" s="36" t="inlineStr">
+      <x:c r="K12" s="36" t="inlineStr">
         <x:is>
           <x:t>后5</x:t>
         </x:is>
       </x:c>
-      <x:c r="L11" s="36" t="inlineStr">
-        <x:is>
-          <x:t>—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M11" s="36" t="str"/>
-    </x:row>
-    <x:row r="12" ht="18" customHeight="1">
-      <x:c r="A12" s="46" t="inlineStr">
-        <x:is>
-          <x:t>【V1.1 · 系统管理控制台（若依风格11页）】（第 5-7 月 · 后5+前1）</x:t>
+      <x:c r="L12" s="36" t="inlineStr">
+        <x:is>
+          <x:t>—</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M12" s="36" t="inlineStr">
+        <x:is>
+          <x:t>基于若依@DataScope；废弃org_id多组织</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -10509,7 +10558,7 @@
       </x:c>
       <x:c r="E13" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F13" s="36" t="inlineStr">
@@ -10574,7 +10623,7 @@
       </x:c>
       <x:c r="E14" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F14" s="36" t="inlineStr">
@@ -10639,7 +10688,7 @@
       </x:c>
       <x:c r="E15" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F15" s="36" t="inlineStr">
@@ -10704,7 +10753,7 @@
       </x:c>
       <x:c r="E16" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F16" s="36" t="inlineStr">
@@ -10769,7 +10818,7 @@
       </x:c>
       <x:c r="E17" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F17" s="36" t="inlineStr">
@@ -10834,7 +10883,7 @@
       </x:c>
       <x:c r="E18" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F18" s="36" t="inlineStr">
@@ -10899,7 +10948,7 @@
       </x:c>
       <x:c r="E19" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F19" s="36" t="inlineStr">
@@ -10964,7 +11013,7 @@
       </x:c>
       <x:c r="E20" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F20" s="36" t="inlineStr">
@@ -11029,7 +11078,7 @@
       </x:c>
       <x:c r="E21" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F21" s="36" t="inlineStr">
@@ -11094,7 +11143,7 @@
       </x:c>
       <x:c r="E22" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F22" s="36" t="inlineStr">
@@ -11159,7 +11208,7 @@
       </x:c>
       <x:c r="E23" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F23" s="36" t="inlineStr">
@@ -11214,7 +11263,7 @@
       </x:c>
       <x:c r="C24" s="36" t="inlineStr">
         <x:is>
-          <x:t>组织与成员管理</x:t>
+          <x:t>部门与成员管理（若依原生）</x:t>
         </x:is>
       </x:c>
       <x:c r="D24" s="36" t="inlineStr">
@@ -11224,12 +11273,12 @@
       </x:c>
       <x:c r="E24" s="36" t="inlineStr">
         <x:is>
-          <x:t>V1.1</x:t>
+          <x:t>V1.0</x:t>
         </x:is>
       </x:c>
       <x:c r="F24" s="36" t="inlineStr">
         <x:is>
-          <x:t>组织CRUD+成员管理</x:t>
+          <x:t>若依原生 sys_dept 部门树 + sys_user 成员管理</x:t>
         </x:is>
       </x:c>
       <x:c r="G24" s="36" t="inlineStr">
@@ -11347,7 +11396,7 @@
       </x:c>
       <x:c r="C27" s="36" t="inlineStr">
         <x:is>
-          <x:t>6角色×21权限完整RBAC</x:t>
+          <x:t>完整角色权限+数据权限（若依深化）</x:t>
         </x:is>
       </x:c>
       <x:c r="D27" s="36" t="inlineStr">
@@ -11362,7 +11411,7 @@
       </x:c>
       <x:c r="F27" s="36" t="inlineStr">
         <x:is>
-          <x:t>完整RBAC权限矩阵</x:t>
+          <x:t>若依完整 RBAC：多角色 + 细粒度菜单/按钮权限点 + @PreAuthorize 注解 + @DataScope 数据权限全套</x:t>
         </x:is>
       </x:c>
       <x:c r="G27" s="36" t="inlineStr">
@@ -11395,17 +11444,16 @@
       </x:c>
       <x:c r="M27" s="36" t="inlineStr">
         <x:is>
-          <x:t>6角色×21权限</x:t>
+          <x:t>基于若依完整RBAC</x:t>
         </x:is>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:mergeCells count="5">
+  <x:mergeCells count="4">
+    <x:mergeCell ref="A4:M4"/>
+    <x:mergeCell ref="A2:M2"/>
     <x:mergeCell ref="A1:M1"/>
-    <x:mergeCell ref="A12:M12"/>
-    <x:mergeCell ref="A4:M4"/>
     <x:mergeCell ref="A25:M25"/>
-    <x:mergeCell ref="A2:M2"/>
   </x:mergeCells>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <x:pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-20 17:56:10
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/MVP功能清单.xlsx
+++ b/公司项目/认知作战/文档/MVP功能清单.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:workbookPr/>
   <x:bookViews>
     <x:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12420" tabRatio="600" firstSheet="1" activeTab="7" autoFilterDateGrouping="1"/>
@@ -1552,7 +1552,7 @@
     </x:row>
     <x:row r="12" ht="55" customHeight="1">
       <x:c r="A12" s="63" t="str">
-        <x:v>V1.0=可演示最小闭环+系统管理控制台（演示主链路+COM若依11页，第1-4月，33页+后端执行链）；V1.1=线框图补齐（第5-7月，10页：MC 6+OCC评估1+SWM评测3）；V1.2=后台增强（第8-10月，桌面端/指标告警/调度/情报分析）；V1.3=深化（第11-12月，IRS多模型/OCC策略库内容图谱Flowable/完整RBAC）。共 12 月 · 6 人（后端5+前端1）。</x:v>
+        <x:v>V1.0=可演示最小闭环+系统管理控制台+完整RBAC（演示主链路+COM若依全套，第1-4月，33页+后端执行链）；V1.1=线框图补齐（第5-7月，10页：MC 6+OCC评估1+SWM评测3）；V1.2=后台增强（第8-10月，桌面端/指标告警/调度/情报分析）；V1.3=深化（第11-12月，IRS多模型/OCC策略库内容图谱Flowable）。共 12 月 · 6 人（后端5+前端1）。COM 全部能力（登录+系统管理11页+完整RBAC）一次性在 V1.0 完成。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
@@ -1859,7 +1859,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="4" ht="90" customHeight="1">
+    <x:row r="4" ht="120" customHeight="1">
       <x:c r="A4" s="53" t="inlineStr">
         <x:is>
           <x:t>第0阶段·地基</x:t>
@@ -1876,7 +1876,7 @@
         </x:is>
       </x:c>
       <x:c r="D4" s="53" t="str">
-        <x:v>COM若依原生登录(/login+/getInfo+/getRouters)+Token签发+Redis共享校验+跨控制台SSO；系统管理控制台11页(若依原生：用户/角色/部门/登录策略/登录日志/菜单/岗位/字典/参数/通知/操作日志)+部门成员管理；开发环境搭建(K8s/PG/Redis/MinIO)；前端骨架(登录/门户)；MC真机ADB接入打通1台</x:v>
+        <x:v>COM若依原生登录(/login+/getInfo+/getRouters)+Token签发+Redis共享校验+跨控制台SSO；完整RBAC(@PreAuthorize+@DataScope全套)；系统管理控制台11页(若依原生：用户/角色/部门/登录策略/登录日志/菜单/岗位/字典/参数/通知/操作日志)+部门成员管理；5次锁定策略+令牌黑名单；开发环境搭建(K8s/PG/Redis/MinIO)；前端骨架(登录/门户)；MC真机ADB接入打通1台</x:v>
       </x:c>
       <x:c r="E4" s="53" t="str">
         <x:v>后5(COM登录+系统管理11页)+前1(骨架+11页)；后1(MC ADB打通)</x:v>
@@ -2055,15 +2055,11 @@
           <x:t>M6：深化</x:t>
         </x:is>
       </x:c>
-      <x:c r="D10" s="58" t="inlineStr">
-        <x:is>
-          <x:t>IRS多模型管理/监控/配额/回退；OCC策略库/内容管理/NebulaGraph图谱/Flowable完整编排；COM完整RBAC(6角色×21权限)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="58" t="inlineStr">
-        <x:is>
-          <x:t>后3(IRS)+后4(OCC深化)+后5(COM RBAC)</x:t>
-        </x:is>
+      <x:c r="D10" s="58" t="str">
+        <x:v>IRS多模型管理/监控/配额/回退；OCC策略库/内容管理/NebulaGraph图谱/Flowable完整编排</x:v>
+      </x:c>
+      <x:c r="E10" s="58" t="str">
+        <x:v>后3(IRS)+后4(OCC深化)</x:v>
       </x:c>
       <x:c r="F10" s="58" t="inlineStr">
         <x:is>
@@ -2624,15 +2620,13 @@
         </x:is>
       </x:c>
       <x:c r="E9" s="36" t="str">
-        <x:v>若依原生登录(/login+/getInfo+/getRouters)；有状态Token(uuid+Base64存Redis)；各子系统查共享Redis校验；跨4控制台SSO；1-2角色(sys_role)；部门数据权限(@DataScope)；5横切页(G-01~05)；系统管理控制台11页(若依原生：用户/角色/部门/登录策略/登录日志/菜单/岗位/字典/参数/通知/操作日志)+部门成员管理</x:v>
+        <x:v>若依原生登录(/login+/getInfo+/getRouters)；有状态Token(uuid+Base64存Redis)；各子系统查共享Redis校验；跨4控制台SSO；完整RBAC(多角色+菜单/按钮权限点+@PreAuthorize+@DataScope全套)；5横切页(G-01~05)；系统管理控制台11页(若依原生：用户/角色/部门/登录策略/登录日志/菜单/岗位/字典/参数/通知/操作日志)+部门成员管理；5次锁定策略+令牌黑名单</x:v>
       </x:c>
       <x:c r="F9" s="36" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="G9" s="36" t="inlineStr">
-        <x:is>
-          <x:t>若依完整RBAC：多角色+细粒度菜单/按钮权限点+@PreAuthorize+@DataScope全套；5次锁定策略；令牌黑名单/登出吊毁</x:t>
-        </x:is>
+      <x:c r="G9" s="36" t="str">
+        <x:v>—</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="110" customHeight="1">
@@ -3587,10 +3581,8 @@
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F17" s="35" t="inlineStr">
-        <x:is>
-          <x:t>代理IP固定绑定（简化）</x:t>
-        </x:is>
+      <x:c r="F17" s="35" t="str">
+        <x:v>终端风控分级+代理绑定（写 mc_binding 网络层侧面 terminal_id+proxy_id）</x:v>
       </x:c>
       <x:c r="G17" s="35" t="inlineStr">
         <x:is>
@@ -3776,10 +3768,8 @@
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F20" s="78" t="inlineStr">
-        <x:is>
-          <x:t>真机绑定固定代理IP（核心逻辑）</x:t>
-        </x:is>
+      <x:c r="F20" s="78" t="str">
+        <x:v>真机绑定固定代理IP，写 mc_binding(terminal_id+proxy_id) 单一存储</x:v>
       </x:c>
       <x:c r="G20" s="78" t="inlineStr">
         <x:is>
@@ -3809,10 +3799,8 @@
           <x:t>MC-05(V1.1)</x:t>
         </x:is>
       </x:c>
-      <x:c r="M20" s="36" t="inlineStr">
-        <x:is>
-          <x:t>一设备一账号一IP；MC-05管理页V1.1</x:t>
-        </x:is>
+      <x:c r="M20" s="36" t="str">
+        <x:v>一设备一账号一IP；写mc_binding单一存储；MC-05管理页V1.1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="40" customHeight="1">
@@ -4676,10 +4664,8 @@
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F34" s="35" t="inlineStr">
-        <x:is>
-          <x:t>四元绑定(简化只读)</x:t>
-        </x:is>
+      <x:c r="F34" s="35" t="str">
+        <x:v>四元绑定(agent_id+account_id+terminal_id+proxy_id)读写，单一存储 mc_binding</x:v>
       </x:c>
       <x:c r="G34" s="35" t="inlineStr">
         <x:is>
@@ -4739,10 +4725,8 @@
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F35" s="78" t="inlineStr">
-        <x:is>
-          <x:t>绑定记录</x:t>
-        </x:is>
+      <x:c r="F35" s="78" t="str">
+        <x:v>agent_id↔account_id 1:1 绑定，写 mc_binding(agent_id+account_id)</x:v>
       </x:c>
       <x:c r="G35" s="78" t="inlineStr">
         <x:is>
@@ -4754,10 +4738,8 @@
           <x:t>全栈</x:t>
         </x:is>
       </x:c>
-      <x:c r="I35" s="36" t="inlineStr">
-        <x:is>
-          <x:t>F-MC-11-01</x:t>
-        </x:is>
+      <x:c r="I35" s="36" t="str">
+        <x:v>F-MC-09-02</x:v>
       </x:c>
       <x:c r="J35" s="36" t="n">
         <x:v>5</x:v>
@@ -4789,10 +4771,8 @@
           <x:t>F-MC-13-02</x:t>
         </x:is>
       </x:c>
-      <x:c r="C36" s="36" t="inlineStr">
-        <x:is>
-          <x:t>四元绑定关系维护</x:t>
-        </x:is>
+      <x:c r="C36" s="36" t="str">
+        <x:v>四元绑定解析（读单一存储）</x:v>
       </x:c>
       <x:c r="D36" s="36" t="inlineStr">
         <x:is>
@@ -4804,10 +4784,8 @@
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F36" s="78" t="inlineStr">
-        <x:is>
-          <x:t>四元绑定只读</x:t>
-        </x:is>
+      <x:c r="F36" s="78" t="str">
+        <x:v>四元行动单元查询/解析，读 mc_binding 单一存储（QuadBindingResolver）；1:1:1:1</x:v>
       </x:c>
       <x:c r="G36" s="78" t="inlineStr">
         <x:is>
@@ -4837,10 +4815,8 @@
           <x:t>MC-21</x:t>
         </x:is>
       </x:c>
-      <x:c r="M36" s="36" t="inlineStr">
-        <x:is>
-          <x:t>V1.0不做维护操作</x:t>
-        </x:is>
+      <x:c r="M36" s="36" t="str">
+        <x:v>读mc_binding单一存储；CON-13 1:1:1:1</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="40" customHeight="1">
@@ -4932,10 +4908,8 @@
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F38" s="78" t="inlineStr">
-        <x:is>
-          <x:t>简化绑定</x:t>
-        </x:is>
+      <x:c r="F38" s="78" t="str">
+        <x:v>账号-终端-代理绑定自动化（BindingAutomator），写 mc_binding(account_id+terminal_id+proxy_id) 单一存储</x:v>
       </x:c>
       <x:c r="G38" s="78" t="inlineStr">
         <x:is>
@@ -4965,10 +4939,8 @@
           <x:t>—</x:t>
         </x:is>
       </x:c>
-      <x:c r="M38" s="36" t="inlineStr">
-        <x:is>
-          <x:t>手动绑定即可</x:t>
-        </x:is>
+      <x:c r="M38" s="36" t="str">
+        <x:v>写mc_binding单一存储；CON-13差异化绑定</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="40" customHeight="1">
@@ -10024,7 +9996,7 @@
     </x:row>
     <x:row r="4" ht="40" customHeight="1">
       <x:c r="A4" s="9" t="str">
-        <x:v>【V1.0 · 登录底座 + 系统管理控制台】（第 1-4 月 · 后5+前1）</x:v>
+        <x:v>【V1.0 · 登录底座 + 系统管理控制台 + 完整RBAC】（第 1-4 月 · 后5+前1）</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
@@ -11312,9 +11284,65 @@
       <x:c r="M24" s="36" t="str"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="51" t="inlineStr">
-        <x:is>
-          <x:t>【V1.3 · 完整RBAC深化】（第 11-12 月 · 后5）</x:t>
+      <x:c r="A25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>③功能</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>F-COM-01-02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>5次锁定策略+令牌黑名单</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>R-COM-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="36" t="str">
+        <x:v>V1.0</x:v>
+      </x:c>
+      <x:c r="F25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>5次锁定+令牌黑名单/登出吊毁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>P2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>后端模块</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>F-COM-01-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J25" s="36" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>后5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>—</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M25" s="36" t="inlineStr">
+        <x:is>
+          <x:t>完整RBAC</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -11326,12 +11354,12 @@
       </x:c>
       <x:c r="B26" s="36" t="inlineStr">
         <x:is>
-          <x:t>F-COM-01-02</x:t>
+          <x:t>F-COM-02-04</x:t>
         </x:is>
       </x:c>
       <x:c r="C26" s="36" t="inlineStr">
         <x:is>
-          <x:t>5次锁定策略+令牌黑名单</x:t>
+          <x:t>完整角色权限+数据权限（若依深化）</x:t>
         </x:is>
       </x:c>
       <x:c r="D26" s="36" t="inlineStr">
@@ -11339,14 +11367,12 @@
           <x:t>R-COM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="E26" s="36" t="inlineStr">
-        <x:is>
-          <x:t>V1.3</x:t>
-        </x:is>
+      <x:c r="E26" s="36" t="str">
+        <x:v>V1.0</x:v>
       </x:c>
       <x:c r="F26" s="36" t="inlineStr">
         <x:is>
-          <x:t>5次锁定+令牌黑名单/登出吊毁</x:t>
+          <x:t>若依完整 RBAC：多角色 + 细粒度菜单/按钮权限点 + @PreAuthorize 注解 + @DataScope 数据权限全套</x:t>
         </x:is>
       </x:c>
       <x:c r="G26" s="36" t="inlineStr">
@@ -11361,11 +11387,11 @@
       </x:c>
       <x:c r="I26" s="36" t="inlineStr">
         <x:is>
-          <x:t>F-COM-01-01</x:t>
+          <x:t>F-COM-02-01</x:t>
         </x:is>
       </x:c>
       <x:c r="J26" s="36" t="n">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="K26" s="36" t="inlineStr">
         <x:is>
@@ -11378,71 +11404,6 @@
         </x:is>
       </x:c>
       <x:c r="M26" s="36" t="inlineStr">
-        <x:is>
-          <x:t>完整RBAC</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>③功能</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>F-COM-02-04</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>完整角色权限+数据权限（若依深化）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>R-COM-001</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>V1.3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>若依完整 RBAC：多角色 + 细粒度菜单/按钮权限点 + @PreAuthorize 注解 + @DataScope 数据权限全套</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>P2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>后端模块</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>F-COM-02-01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J27" s="36" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="K27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>后5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L27" s="36" t="inlineStr">
-        <x:is>
-          <x:t>—</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M27" s="36" t="inlineStr">
         <x:is>
           <x:t>基于若依完整RBAC</x:t>
         </x:is>
@@ -11453,7 +11414,6 @@
     <x:mergeCell ref="A4:M4"/>
     <x:mergeCell ref="A2:M2"/>
     <x:mergeCell ref="A1:M1"/>
-    <x:mergeCell ref="A25:M25"/>
   </x:mergeCells>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <x:pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-20 18:06:19
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/MVP功能清单.xlsx
+++ b/公司项目/认知作战/文档/MVP功能清单.xlsx
@@ -2481,10 +2481,8 @@
           <x:t>评测闭环：评测集/评估器/实验/评估打分(M-SWM-06)；版本输出对比。3页(SWM-06/07/08)</x:t>
         </x:is>
       </x:c>
-      <x:c r="G5" s="36" t="inlineStr">
-        <x:is>
-          <x:t>记忆沉淀/个性化延续；迭代决策；swm-distill提炼编排</x:t>
-        </x:is>
+      <x:c r="G5" s="36" t="str">
+        <x:v>记忆沉淀/个性化延续（按account_id）；迭代决策；swm-distill提炼编排</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="110" customHeight="1">
@@ -4665,7 +4663,7 @@
         </x:is>
       </x:c>
       <x:c r="F34" s="35" t="str">
-        <x:v>四元绑定(agent_id+account_id+terminal_id+proxy_id)读写，单一存储 mc_binding</x:v>
+        <x:v>行动关系(agent_id+account_id+terminal_id+proxy_id)读写，单一存储 mc_binding；agent:账号=1:N，账号:终端:IP=1:1:1</x:v>
       </x:c>
       <x:c r="G34" s="35" t="inlineStr">
         <x:is>
@@ -4693,10 +4691,8 @@
         </x:is>
       </x:c>
       <x:c r="L34" s="10" t="str"/>
-      <x:c r="M34" s="10" t="inlineStr">
-        <x:is>
-          <x:t>agent_id:account:终端:IP</x:t>
-        </x:is>
+      <x:c r="M34" s="10" t="str">
+        <x:v>agent:account:终端:IP = 1:N:1:1</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="40" customHeight="1">
@@ -4726,7 +4722,7 @@
         </x:is>
       </x:c>
       <x:c r="F35" s="78" t="str">
-        <x:v>agent_id↔account_id 1:1 绑定，写 mc_binding(agent_id+account_id)</x:v>
+        <x:v>agent_id↔account_id 1:N 绑定（一个agent绑多账号），写 mc_binding(agent_id+account_id)；账号级记忆/动态提示词按 account_id 1:1 归属</x:v>
       </x:c>
       <x:c r="G35" s="78" t="inlineStr">
         <x:is>
@@ -4754,10 +4750,8 @@
           <x:t>MC-21</x:t>
         </x:is>
       </x:c>
-      <x:c r="M35" s="36" t="inlineStr">
-        <x:is>
-          <x:t>1:1</x:t>
-        </x:is>
+      <x:c r="M35" s="36" t="str">
+        <x:v>1:N</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="40" customHeight="1">
@@ -4785,7 +4779,7 @@
         </x:is>
       </x:c>
       <x:c r="F36" s="78" t="str">
-        <x:v>四元行动单元查询/解析，读 mc_binding 单一存储（QuadBindingResolver）；1:1:1:1</x:v>
+        <x:v>行动关系查询/解析，读 mc_binding 单一存储（BindingResolver）；1:N:1:1</x:v>
       </x:c>
       <x:c r="G36" s="78" t="inlineStr">
         <x:is>
@@ -4816,7 +4810,7 @@
         </x:is>
       </x:c>
       <x:c r="M36" s="36" t="str">
-        <x:v>读mc_binding单一存储；CON-13 1:1:1:1</x:v>
+        <x:v>读mc_binding单一存储；CON-13 1:N:1:1</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="40" customHeight="1">
@@ -7474,10 +7468,8 @@
           <x:t>F-MC-13-03</x:t>
         </x:is>
       </x:c>
-      <x:c r="C81" s="36" t="inlineStr">
-        <x:is>
-          <x:t>迁移资产抽取</x:t>
-        </x:is>
+      <x:c r="C81" s="36" t="str">
+        <x:v>账号资产抽取</x:v>
       </x:c>
       <x:c r="D81" s="36" t="inlineStr">
         <x:is>
@@ -7535,10 +7527,8 @@
           <x:t>F-MC-13-04</x:t>
         </x:is>
       </x:c>
-      <x:c r="C82" s="36" t="inlineStr">
-        <x:is>
-          <x:t>迁移目标账号校验</x:t>
-        </x:is>
+      <x:c r="C82" s="36" t="str">
+        <x:v>迁移目标账号校验</x:v>
       </x:c>
       <x:c r="D82" s="36" t="inlineStr">
         <x:is>
@@ -12126,10 +12116,8 @@
           <x:t>V1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="F14" s="78" t="inlineStr">
-        <x:is>
-          <x:t>基础记忆存储</x:t>
-        </x:is>
+      <x:c r="F14" s="78" t="str">
+        <x:v>基础记忆存储（account_id 主键，账号级 1:1）</x:v>
       </x:c>
       <x:c r="G14" s="78" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
vault backup: 2026-07-21 11:28:27
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/MVP功能清单.xlsx
+++ b/公司项目/认知作战/文档/MVP功能清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="32400" windowHeight="17820" firstSheet="1" activeTab="2"/>
+    <workbookView windowWidth="32400" windowHeight="17820" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="说明" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2610" uniqueCount="1012">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2609" uniqueCount="1012">
   <si>
     <t>认知行动平台 · 功能清单（V1.0~V1.3）</t>
   </si>
@@ -342,7 +342,27 @@
     <t>MC 多设备矩阵自动化群控子系统 · 功能清单（V1.0~V1.3）</t>
   </si>
   <si>
-    <t>按模块→功能层级，分版本（V1.0 演示主链路 / V1.1 线框图补齐 / V1.2 后台增强 / V1.3 深化），行序按依赖重排（前置依赖在前）。优先级：P0=必做 / P1=应做 / P2=可缓。类型：后端模块 / 前端页 / 全栈。工期单位=人天。完成人：后1=MC执行链 / 后2=MC业务链 / 前1=前端。</t>
+    <r>
+      <t>排期选取最大工作日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> 26</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>天</t>
+    </r>
   </si>
   <si>
     <t>层级</t>
@@ -1173,9 +1193,6 @@
     <t>全量动作留痕</t>
   </si>
   <si>
-    <t>郝宇</t>
-  </si>
-  <si>
     <t>F-MC-10-02</t>
   </si>
   <si>
@@ -2131,6 +2148,101 @@
     <t>COM 公共功能 · 功能清单（V1.0~V1.3）</t>
   </si>
   <si>
+    <r>
+      <t>按模块</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>功能层级，分版本（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>V1.0~V1.3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>），行序按依赖重排。完成人：后</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">5=COM+DC+OM / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>前</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>1=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>前端。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="22"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>涉及到微服务整体架构部署</t>
+    </r>
+  </si>
+  <si>
     <t>【V1.0 · 登录底座 + 系统管理控制台 + 完整RBAC】（第 1-4 月 · 后5+前1）</t>
   </si>
   <si>
@@ -3527,7 +3639,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -3585,6 +3697,12 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Noto Serif CJK SC"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF595959"/>
       <name val="Noto Serif CJK SC"/>
       <charset val="134"/>
     </font>
@@ -3794,6 +3912,12 @@
       <b/>
       <sz val="16"/>
       <color rgb="FF1F4E79"/>
+      <name val="Noto Serif CJK SC"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="22"/>
+      <color rgb="FFFF0000"/>
       <name val="Noto Serif CJK SC"/>
       <charset val="134"/>
     </font>
@@ -4137,31 +4261,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="18" fillId="0" borderId="0">
+    <xf numFmtId="43" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="18" fillId="0" borderId="0">
+    <xf numFmtId="44" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="18" fillId="0" borderId="0">
+    <xf numFmtId="9" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="18" fillId="0" borderId="0">
+    <xf numFmtId="41" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="18" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
+    <xf numFmtId="42" fontId="19" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
@@ -4170,119 +4291,122 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="4">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="5">
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="4">
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="6">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="8">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="7">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="3" borderId="0">
+    <xf numFmtId="0" fontId="34" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="35" fillId="3" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="34" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="36" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="37" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="38" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4348,16 +4472,22 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4366,19 +4496,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4391,10 +4521,10 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -4798,65 +4928,65 @@
   </cols>
   <sheetData>
     <row r="1" ht="23.25" customHeight="1" spans="1:2">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:2">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="36" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:2">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="38" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:2">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="38" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:2">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="38" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="37">
+      <c r="B7" s="39">
         <v>46223</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:2">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="38" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:2">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="40" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" ht="55" customHeight="1" spans="1:2">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="38" t="s">
         <v>12</v>
       </c>
     </row>
@@ -4866,7 +4996,7 @@
       </c>
     </row>
     <row r="12" ht="55" customHeight="1" spans="1:2">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="41" t="s">
         <v>14</v>
       </c>
     </row>
@@ -4876,17 +5006,17 @@
       </c>
     </row>
     <row r="14" ht="55" customHeight="1" spans="1:2">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="38" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:2">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="40" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" ht="55" customHeight="1" spans="1:2">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="38" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4896,7 +5026,7 @@
       </c>
     </row>
     <row r="18" ht="25" customHeight="1" spans="1:3">
-      <c r="A18" s="39" t="s">
+      <c r="A18" s="41" t="s">
         <v>20</v>
       </c>
     </row>
@@ -4906,20 +5036,20 @@
       </c>
     </row>
     <row r="20" ht="25" customHeight="1" spans="1:3">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="38" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:3">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="40" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="22" ht="40" customHeight="1" spans="1:3">
-      <c r="A22" s="35" t="s">
+      <c r="A22" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="40"/>
+      <c r="C22" s="42"/>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:3">
       <c r="A23" s="21" t="s">
@@ -4927,34 +5057,34 @@
       </c>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:3">
-      <c r="A24" s="36" t="s">
+      <c r="A24" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="38" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:3">
-      <c r="A25" s="36" t="s">
+      <c r="A25" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="36" t="s">
+      <c r="B25" s="38" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:3">
-      <c r="A26" s="36" t="s">
+      <c r="A26" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="36" t="s">
+      <c r="B26" s="38" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:3">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="36" t="s">
+      <c r="B27" s="38" t="s">
         <v>33</v>
       </c>
       <c r="C27">
@@ -4962,10 +5092,10 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:3">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="36" t="s">
+      <c r="B28" s="38" t="s">
         <v>35</v>
       </c>
       <c r="C28">
@@ -4973,10 +5103,10 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1" spans="1:3">
-      <c r="A29" s="36" t="s">
+      <c r="A29" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="38" t="s">
         <v>37</v>
       </c>
       <c r="C29">
@@ -4984,10 +5114,10 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:3">
-      <c r="A30" s="36" t="s">
+      <c r="A30" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="B30" s="36" t="s">
+      <c r="B30" s="38" t="s">
         <v>39</v>
       </c>
       <c r="C30">
@@ -4995,10 +5125,10 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1" spans="1:3">
-      <c r="A31" s="36" t="s">
+      <c r="A31" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="36" t="s">
+      <c r="B31" s="38" t="s">
         <v>41</v>
       </c>
       <c r="C31">
@@ -5006,10 +5136,10 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:3">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="B32" s="36" t="s">
+      <c r="B32" s="38" t="s">
         <v>43</v>
       </c>
       <c r="C32">
@@ -5017,10 +5147,10 @@
       </c>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:2">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="B33" s="36" t="s">
+      <c r="B33" s="38" t="s">
         <v>45</v>
       </c>
     </row>
@@ -5676,7 +5806,7 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1" spans="1:14">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="23" t="s">
         <v>101</v>
       </c>
     </row>
@@ -5684,7 +5814,7 @@
       <c r="A3" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="25" t="s">
         <v>103</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -5737,7 +5867,7 @@
       <c r="C5" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="26" t="s">
         <v>119</v>
       </c>
       <c r="E5" s="14" t="s">
@@ -5775,7 +5905,7 @@
       <c r="A6" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="27" t="s">
         <v>126</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -5912,7 +6042,7 @@
       <c r="F9" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="G9" s="25" t="s">
+      <c r="G9" s="27" t="s">
         <v>143</v>
       </c>
       <c r="H9" s="16" t="s">
@@ -5981,7 +6111,7 @@
       <c r="C11" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="26" t="s">
         <v>150</v>
       </c>
       <c r="E11" s="14" t="s">
@@ -6017,7 +6147,7 @@
       <c r="A12" t="s">
         <v>125</v>
       </c>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="28" t="s">
         <v>154</v>
       </c>
       <c r="C12" t="s">
@@ -6044,7 +6174,7 @@
       <c r="J12" t="s">
         <v>127</v>
       </c>
-      <c r="K12" s="27">
+      <c r="K12" s="29">
         <v>14</v>
       </c>
       <c r="L12" t="s">
@@ -6058,7 +6188,7 @@
       <c r="A13" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="28"/>
+      <c r="B13" s="30"/>
       <c r="C13" t="s">
         <v>160</v>
       </c>
@@ -6083,7 +6213,7 @@
       <c r="J13" t="s">
         <v>155</v>
       </c>
-      <c r="K13" s="27"/>
+      <c r="K13" s="29"/>
       <c r="L13" t="s">
         <v>158</v>
       </c>
@@ -6098,7 +6228,7 @@
       <c r="A14" t="s">
         <v>125</v>
       </c>
-      <c r="B14" s="28"/>
+      <c r="B14" s="30"/>
       <c r="C14" t="s">
         <v>165</v>
       </c>
@@ -6123,7 +6253,7 @@
       <c r="J14" t="s">
         <v>155</v>
       </c>
-      <c r="K14" s="27"/>
+      <c r="K14" s="29"/>
       <c r="L14" t="s">
         <v>158</v>
       </c>
@@ -6135,7 +6265,7 @@
       <c r="A15" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="30"/>
       <c r="C15" t="s">
         <v>169</v>
       </c>
@@ -6160,7 +6290,7 @@
       <c r="J15" t="s">
         <v>155</v>
       </c>
-      <c r="K15" s="27"/>
+      <c r="K15" s="29"/>
       <c r="L15" t="s">
         <v>158</v>
       </c>
@@ -6172,7 +6302,7 @@
       <c r="A16" t="s">
         <v>125</v>
       </c>
-      <c r="B16" s="28"/>
+      <c r="B16" s="30"/>
       <c r="C16" t="s">
         <v>173</v>
       </c>
@@ -6197,7 +6327,7 @@
       <c r="J16" t="s">
         <v>155</v>
       </c>
-      <c r="K16" s="27"/>
+      <c r="K16" s="29"/>
       <c r="L16" t="s">
         <v>158</v>
       </c>
@@ -6209,7 +6339,7 @@
       <c r="A17" t="s">
         <v>125</v>
       </c>
-      <c r="B17" s="28"/>
+      <c r="B17" s="30"/>
       <c r="C17" t="s">
         <v>177</v>
       </c>
@@ -6222,7 +6352,7 @@
       <c r="F17" t="s">
         <v>121</v>
       </c>
-      <c r="G17" s="25" t="s">
+      <c r="G17" s="27" t="s">
         <v>179</v>
       </c>
       <c r="H17" t="s">
@@ -6234,7 +6364,7 @@
       <c r="J17" t="s">
         <v>165</v>
       </c>
-      <c r="K17" s="27"/>
+      <c r="K17" s="29"/>
       <c r="L17" t="s">
         <v>158</v>
       </c>
@@ -6291,7 +6421,7 @@
       <c r="A19" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="27" t="s">
         <v>187</v>
       </c>
       <c r="C19" s="4" t="s">
@@ -6318,7 +6448,9 @@
       <c r="J19" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K19" s="16"/>
+      <c r="K19" s="16">
+        <v>7</v>
+      </c>
       <c r="L19" s="18" t="s">
         <v>192</v>
       </c>
@@ -6602,8 +6734,8 @@
       <c r="J26" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="K26" s="4">
-        <v>8</v>
+      <c r="K26" s="16">
+        <v>5</v>
       </c>
       <c r="L26" s="18" t="s">
         <v>192</v>
@@ -6638,15 +6770,13 @@
       <c r="H27" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="I27" s="29" t="s">
+      <c r="I27" s="31" t="s">
         <v>123</v>
       </c>
       <c r="J27" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="K27" s="4">
-        <v>8</v>
-      </c>
+      <c r="K27" s="16"/>
       <c r="L27" s="18" t="s">
         <v>192</v>
       </c>
@@ -6703,7 +6833,7 @@
       <c r="A29" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B29" s="25" t="s">
+      <c r="B29" s="27" t="s">
         <v>154</v>
       </c>
       <c r="C29" s="4" t="s">
@@ -6730,8 +6860,8 @@
       <c r="J29" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="K29" s="4">
-        <v>15</v>
+      <c r="K29" s="16">
+        <v>7</v>
       </c>
       <c r="L29" t="s">
         <v>158</v>
@@ -6772,9 +6902,7 @@
       <c r="J30" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="K30" s="4">
-        <v>10</v>
-      </c>
+      <c r="K30" s="16"/>
       <c r="L30" t="s">
         <v>158</v>
       </c>
@@ -6831,7 +6959,7 @@
       <c r="A32" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B32" s="25" t="s">
+      <c r="B32" s="27" t="s">
         <v>187</v>
       </c>
       <c r="C32" s="4" t="s">
@@ -6858,8 +6986,8 @@
       <c r="J32" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K32" s="4">
-        <v>13</v>
+      <c r="K32" s="16">
+        <v>14</v>
       </c>
       <c r="L32" s="18" t="s">
         <v>131</v>
@@ -6900,9 +7028,7 @@
       <c r="J33" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K33" s="4">
-        <v>15</v>
-      </c>
+      <c r="K33" s="16"/>
       <c r="L33" s="18" t="s">
         <v>131</v>
       </c>
@@ -6986,8 +7112,8 @@
       <c r="J35" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="K35" s="4">
-        <v>10</v>
+      <c r="K35" s="16">
+        <v>5</v>
       </c>
       <c r="L35" s="18" t="s">
         <v>192</v>
@@ -7028,9 +7154,7 @@
       <c r="J36" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="K36" s="4">
-        <v>5</v>
-      </c>
+      <c r="K36" s="16"/>
       <c r="L36" s="18" t="s">
         <v>192</v>
       </c>
@@ -7070,9 +7194,7 @@
       <c r="J37" s="19" t="s">
         <v>273</v>
       </c>
-      <c r="K37" s="4">
-        <v>5</v>
-      </c>
+      <c r="K37" s="16"/>
       <c r="L37" s="18" t="s">
         <v>192</v>
       </c>
@@ -7129,7 +7251,7 @@
       <c r="A39" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="25" t="s">
+      <c r="B39" s="27" t="s">
         <v>286</v>
       </c>
       <c r="C39" s="4" t="s">
@@ -7156,7 +7278,7 @@
       <c r="J39" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="K39" s="4">
+      <c r="K39" s="16">
         <v>5</v>
       </c>
       <c r="L39" s="18" t="s">
@@ -7198,9 +7320,7 @@
       <c r="J40" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="K40" s="4">
-        <v>3</v>
-      </c>
+      <c r="K40" s="16"/>
       <c r="L40" s="18" t="s">
         <v>8</v>
       </c>
@@ -7284,8 +7404,8 @@
       <c r="J42" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K42" s="4">
-        <v>8</v>
+      <c r="K42" s="16">
+        <v>7</v>
       </c>
       <c r="L42" s="18" t="s">
         <v>131</v>
@@ -7326,9 +7446,7 @@
       <c r="J43" s="4" t="s">
         <v>300</v>
       </c>
-      <c r="K43" s="4">
-        <v>5</v>
-      </c>
+      <c r="K43" s="16"/>
       <c r="L43" s="18" t="s">
         <v>131</v>
       </c>
@@ -7368,9 +7486,7 @@
       <c r="J44" s="19" t="s">
         <v>300</v>
       </c>
-      <c r="K44" s="4">
-        <v>8</v>
-      </c>
+      <c r="K44" s="16"/>
       <c r="L44" s="18" t="s">
         <v>131</v>
       </c>
@@ -7410,9 +7526,7 @@
       <c r="J45" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="K45" s="4">
-        <v>3</v>
-      </c>
+      <c r="K45" s="16"/>
       <c r="L45" s="18" t="s">
         <v>131</v>
       </c>
@@ -7469,7 +7583,7 @@
       <c r="A47" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B47" s="25" t="s">
+      <c r="B47" s="27" t="s">
         <v>187</v>
       </c>
       <c r="C47" s="4" t="s">
@@ -7496,11 +7610,11 @@
       <c r="J47" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="K47" s="4">
-        <v>5</v>
+      <c r="K47" s="16">
+        <v>7</v>
       </c>
       <c r="L47" s="18" t="s">
-        <v>322</v>
+        <v>192</v>
       </c>
       <c r="M47" s="4" t="s">
         <v>139</v>
@@ -7515,10 +7629,10 @@
       </c>
       <c r="B48" s="16"/>
       <c r="C48" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="D48" s="4" t="s">
         <v>323</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>324</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>316</v>
@@ -7527,7 +7641,7 @@
         <v>121</v>
       </c>
       <c r="G48" s="16" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H48" s="16" t="s">
         <v>144</v>
@@ -7538,11 +7652,9 @@
       <c r="J48" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="K48" s="4">
-        <v>5</v>
-      </c>
+      <c r="K48" s="16"/>
       <c r="L48" s="18" t="s">
-        <v>322</v>
+        <v>192</v>
       </c>
       <c r="M48" s="4" t="s">
         <v>139</v>
@@ -7557,10 +7669,10 @@
       </c>
       <c r="B49" s="16"/>
       <c r="C49" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="D49" s="4" t="s">
         <v>326</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>327</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>316</v>
@@ -7569,7 +7681,7 @@
         <v>121</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="H49" s="16" t="s">
         <v>144</v>
@@ -7580,11 +7692,9 @@
       <c r="J49" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="K49" s="4">
-        <v>5</v>
-      </c>
+      <c r="K49" s="16"/>
       <c r="L49" s="18" t="s">
-        <v>322</v>
+        <v>192</v>
       </c>
       <c r="M49" s="4" t="s">
         <v>139</v>
@@ -7599,10 +7709,10 @@
       </c>
       <c r="B50" s="16"/>
       <c r="C50" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="D50" s="19" t="s">
         <v>329</v>
-      </c>
-      <c r="D50" s="19" t="s">
-        <v>330</v>
       </c>
       <c r="E50" s="19" t="s">
         <v>316</v>
@@ -7611,7 +7721,7 @@
         <v>121</v>
       </c>
       <c r="G50" s="20" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H50" s="20" t="s">
         <v>130</v>
@@ -7622,17 +7732,15 @@
       <c r="J50" s="19" t="s">
         <v>319</v>
       </c>
-      <c r="K50" s="4">
-        <v>5</v>
-      </c>
+      <c r="K50" s="16"/>
       <c r="L50" s="18" t="s">
-        <v>322</v>
+        <v>192</v>
       </c>
       <c r="M50" s="4" t="s">
         <v>74</v>
       </c>
       <c r="N50" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="51" ht="40" customHeight="1" spans="1:14">
@@ -7641,10 +7749,10 @@
       </c>
       <c r="B51" s="16"/>
       <c r="C51" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="D51" s="4" t="s">
         <v>333</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>334</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>316</v>
@@ -7653,7 +7761,7 @@
         <v>121</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H51" s="16" t="s">
         <v>197</v>
@@ -7662,19 +7770,17 @@
         <v>191</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="K51" s="4">
-        <v>5</v>
-      </c>
+        <v>322</v>
+      </c>
+      <c r="K51" s="16"/>
       <c r="L51" s="18" t="s">
-        <v>322</v>
+        <v>192</v>
       </c>
       <c r="M51" s="4" t="s">
         <v>139</v>
       </c>
       <c r="N51" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="52" ht="40" customHeight="1" spans="1:14">
@@ -7683,19 +7789,19 @@
       </c>
       <c r="B52" s="14"/>
       <c r="C52" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="D52" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="D52" s="14" t="s">
+      <c r="E52" s="14" t="s">
         <v>338</v>
-      </c>
-      <c r="E52" s="14" t="s">
-        <v>339</v>
       </c>
       <c r="F52" s="14" t="s">
         <v>121</v>
       </c>
       <c r="G52" s="15" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H52" s="15" t="s">
         <v>74</v>
@@ -7704,7 +7810,7 @@
         <v>123</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K52" s="14" t="s">
         <v>74</v>
@@ -7716,7 +7822,7 @@
         <v>10</v>
       </c>
       <c r="N52" s="14" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="53" ht="40" customHeight="1" spans="1:14">
@@ -7727,19 +7833,19 @@
         <v>286</v>
       </c>
       <c r="C53" s="19" t="s">
+        <v>342</v>
+      </c>
+      <c r="D53" s="19" t="s">
         <v>343</v>
       </c>
-      <c r="D53" s="19" t="s">
-        <v>344</v>
-      </c>
       <c r="E53" s="19" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F53" s="19" t="s">
         <v>121</v>
       </c>
       <c r="G53" s="20" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H53" s="20" t="s">
         <v>130</v>
@@ -7748,10 +7854,10 @@
         <v>191</v>
       </c>
       <c r="J53" s="19" t="s">
-        <v>341</v>
-      </c>
-      <c r="K53" s="4">
-        <v>8</v>
+        <v>340</v>
+      </c>
+      <c r="K53" s="16">
+        <v>5</v>
       </c>
       <c r="L53" s="18" t="s">
         <v>8</v>
@@ -7760,7 +7866,7 @@
         <v>261</v>
       </c>
       <c r="N53" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="54" ht="40" customHeight="1" spans="1:14">
@@ -7769,19 +7875,19 @@
       </c>
       <c r="B54" s="20"/>
       <c r="C54" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="D54" s="4" t="s">
         <v>347</v>
       </c>
-      <c r="D54" s="4" t="s">
-        <v>348</v>
-      </c>
       <c r="E54" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>121</v>
       </c>
       <c r="G54" s="16" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="H54" s="16" t="s">
         <v>144</v>
@@ -7790,11 +7896,9 @@
         <v>191</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>343</v>
-      </c>
-      <c r="K54" s="4">
-        <v>5</v>
-      </c>
+        <v>342</v>
+      </c>
+      <c r="K54" s="16"/>
       <c r="L54" s="18" t="s">
         <v>8</v>
       </c>
@@ -7802,7 +7906,7 @@
         <v>261</v>
       </c>
       <c r="N54" s="4" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="55" ht="40" customHeight="1" spans="1:14">
@@ -7811,19 +7915,19 @@
       </c>
       <c r="B55" s="20"/>
       <c r="C55" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="D55" s="4" t="s">
         <v>351</v>
       </c>
-      <c r="D55" s="4" t="s">
-        <v>352</v>
-      </c>
       <c r="E55" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>121</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H55" s="16" t="s">
         <v>130</v>
@@ -7832,11 +7936,9 @@
         <v>123</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="K55" s="4">
-        <v>5</v>
-      </c>
+        <v>353</v>
+      </c>
+      <c r="K55" s="16"/>
       <c r="L55" s="18" t="s">
         <v>8</v>
       </c>
@@ -7853,19 +7955,19 @@
       </c>
       <c r="B56" s="20"/>
       <c r="C56" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="D56" s="4" t="s">
         <v>355</v>
       </c>
-      <c r="D56" s="4" t="s">
-        <v>356</v>
-      </c>
       <c r="E56" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F56" s="4" t="s">
         <v>121</v>
       </c>
       <c r="G56" s="16" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="H56" s="16" t="s">
         <v>130</v>
@@ -7874,11 +7976,9 @@
         <v>191</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>358</v>
-      </c>
-      <c r="K56" s="4">
-        <v>5</v>
-      </c>
+        <v>357</v>
+      </c>
+      <c r="K56" s="16"/>
       <c r="L56" s="18" t="s">
         <v>8</v>
       </c>
@@ -7895,10 +7995,10 @@
       </c>
       <c r="B57" s="20"/>
       <c r="C57" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="D57" s="4" t="s">
         <v>359</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>360</v>
       </c>
       <c r="E57" s="4" t="s">
         <v>316</v>
@@ -7907,25 +8007,23 @@
         <v>121</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H57" s="16" t="s">
         <v>144</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J57" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="K57" s="4">
-        <v>8</v>
-      </c>
+      <c r="K57" s="16"/>
       <c r="L57" s="18" t="s">
         <v>8</v>
       </c>
       <c r="M57" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="N57" s="4" t="s">
         <v>314</v>
@@ -7937,19 +8035,19 @@
       </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="D58" s="14" t="s">
         <v>364</v>
       </c>
-      <c r="D58" s="14" t="s">
+      <c r="E58" s="14" t="s">
         <v>365</v>
-      </c>
-      <c r="E58" s="14" t="s">
-        <v>366</v>
       </c>
       <c r="F58" s="14" t="s">
         <v>229</v>
       </c>
       <c r="G58" s="15" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="H58" s="15" t="s">
         <v>74</v>
@@ -7970,7 +8068,7 @@
         <v>10</v>
       </c>
       <c r="N58" s="14" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="59" ht="40" customHeight="1" spans="1:14">
@@ -7981,19 +8079,19 @@
         <v>187</v>
       </c>
       <c r="C59" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="D59" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="D59" s="4" t="s">
-        <v>370</v>
-      </c>
       <c r="E59" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F59" s="4" t="s">
         <v>229</v>
       </c>
       <c r="G59" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H59" s="16" t="s">
         <v>144</v>
@@ -8004,15 +8102,13 @@
       <c r="J59" s="4" t="s">
         <v>300</v>
       </c>
-      <c r="K59" s="4">
-        <v>10</v>
-      </c>
+      <c r="K59" s="16"/>
       <c r="L59" s="18"/>
       <c r="M59" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="N59" s="4" t="s">
         <v>372</v>
-      </c>
-      <c r="N59" s="4" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="60" ht="40" customHeight="1" spans="1:14">
@@ -8021,19 +8117,19 @@
       </c>
       <c r="B60" s="16"/>
       <c r="C60" s="19" t="s">
+        <v>373</v>
+      </c>
+      <c r="D60" s="19" t="s">
         <v>374</v>
       </c>
-      <c r="D60" s="19" t="s">
-        <v>375</v>
-      </c>
       <c r="E60" s="19" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F60" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="G60" s="30" t="s">
-        <v>376</v>
+      <c r="G60" s="32" t="s">
+        <v>375</v>
       </c>
       <c r="H60" s="20" t="s">
         <v>144</v>
@@ -8044,15 +8140,13 @@
       <c r="J60" s="19" t="s">
         <v>253</v>
       </c>
-      <c r="K60" s="4">
-        <v>15</v>
-      </c>
+      <c r="K60" s="16"/>
       <c r="L60" s="18"/>
       <c r="M60" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="N60" s="4" t="s">
         <v>377</v>
-      </c>
-      <c r="N60" s="4" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="61" ht="40" customHeight="1" spans="1:14">
@@ -8061,19 +8155,19 @@
       </c>
       <c r="B61" s="16"/>
       <c r="C61" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D61" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="D61" s="4" t="s">
-        <v>380</v>
-      </c>
       <c r="E61" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>229</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H61" s="16" t="s">
         <v>144</v>
@@ -8082,14 +8176,12 @@
         <v>191</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="K61" s="4">
-        <v>10</v>
-      </c>
+        <v>373</v>
+      </c>
+      <c r="K61" s="16"/>
       <c r="L61" s="18"/>
       <c r="M61" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="N61" s="4" t="s">
         <v>10</v>
@@ -8101,10 +8193,10 @@
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="D62" s="4" t="s">
         <v>383</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>384</v>
       </c>
       <c r="E62" s="4" t="s">
         <v>184</v>
@@ -8113,7 +8205,7 @@
         <v>229</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="H62" s="16" t="s">
         <v>197</v>
@@ -8124,12 +8216,10 @@
       <c r="J62" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="K62" s="4">
-        <v>8</v>
-      </c>
+      <c r="K62" s="16"/>
       <c r="L62" s="18"/>
       <c r="M62" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="N62" s="4" t="s">
         <v>10</v>
@@ -8141,10 +8231,10 @@
       </c>
       <c r="B63" s="16"/>
       <c r="C63" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="D63" s="4" t="s">
         <v>387</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>388</v>
       </c>
       <c r="E63" s="4" t="s">
         <v>297</v>
@@ -8153,7 +8243,7 @@
         <v>229</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H63" s="16" t="s">
         <v>197</v>
@@ -8164,9 +8254,7 @@
       <c r="J63" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="K63" s="4">
-        <v>8</v>
-      </c>
+      <c r="K63" s="16"/>
       <c r="L63" s="18"/>
       <c r="M63" s="4" t="s">
         <v>303</v>
@@ -8181,10 +8269,10 @@
       </c>
       <c r="B64" s="16"/>
       <c r="C64" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="D64" s="4" t="s">
         <v>390</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>391</v>
       </c>
       <c r="E64" s="4" t="s">
         <v>316</v>
@@ -8193,7 +8281,7 @@
         <v>229</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="H64" s="16" t="s">
         <v>197</v>
@@ -8204,9 +8292,7 @@
       <c r="J64" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="K64" s="4">
-        <v>8</v>
-      </c>
+      <c r="K64" s="16"/>
       <c r="L64" s="18"/>
       <c r="M64" s="4" t="s">
         <v>139</v>
@@ -8216,8 +8302,8 @@
       </c>
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:14">
-      <c r="A65" s="31" t="s">
-        <v>393</v>
+      <c r="A65" s="33" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="66" ht="40" customHeight="1" spans="1:14">
@@ -8226,19 +8312,19 @@
       </c>
       <c r="B66" s="4"/>
       <c r="C66" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="D66" s="4" t="s">
         <v>394</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>395</v>
       </c>
       <c r="E66" s="4" t="s">
         <v>184</v>
       </c>
       <c r="F66" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="G66" s="4" t="s">
         <v>396</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>397</v>
       </c>
       <c r="H66" s="16" t="s">
         <v>197</v>
@@ -8257,7 +8343,7 @@
         <v>163</v>
       </c>
       <c r="N66" s="4" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="67" ht="40" customHeight="1" spans="1:14">
@@ -8266,19 +8352,19 @@
       </c>
       <c r="B67" s="4"/>
       <c r="C67" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="D67" s="4" t="s">
         <v>399</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>400</v>
       </c>
       <c r="E67" s="4" t="s">
         <v>206</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H67" s="16" t="s">
         <v>197</v>
@@ -8287,7 +8373,7 @@
         <v>123</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="K67" s="4">
         <v>10</v>
@@ -8297,7 +8383,7 @@
         <v>74</v>
       </c>
       <c r="N67" s="4" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="68" ht="40" customHeight="1" spans="1:14">
@@ -8306,19 +8392,19 @@
       </c>
       <c r="B68" s="4"/>
       <c r="C68" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="D68" s="4" t="s">
         <v>403</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>404</v>
       </c>
       <c r="E68" s="4" t="s">
         <v>201</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="H68" s="16" t="s">
         <v>197</v>
@@ -8327,7 +8413,7 @@
         <v>123</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="K68" s="4">
         <v>13</v>
@@ -8337,7 +8423,7 @@
         <v>74</v>
       </c>
       <c r="N68" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="69" ht="40" customHeight="1" spans="1:14">
@@ -8346,19 +8432,19 @@
       </c>
       <c r="B69" s="4"/>
       <c r="C69" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D69" s="4" t="s">
         <v>407</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>408</v>
       </c>
       <c r="E69" s="4" t="s">
         <v>235</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="H69" s="16" t="s">
         <v>197</v>
@@ -8367,7 +8453,7 @@
         <v>191</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="K69" s="4">
         <v>10</v>
@@ -8377,7 +8463,7 @@
         <v>180</v>
       </c>
       <c r="N69" s="4" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="70" ht="40" customHeight="1" spans="1:14">
@@ -8386,19 +8472,19 @@
       </c>
       <c r="B70" s="4"/>
       <c r="C70" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="D70" s="4" t="s">
         <v>410</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>411</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>235</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="H70" s="16" t="s">
         <v>197</v>
@@ -8426,19 +8512,19 @@
       </c>
       <c r="B71" s="4"/>
       <c r="C71" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>412</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>413</v>
       </c>
       <c r="E71" s="4" t="s">
         <v>211</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H71" s="16" t="s">
         <v>197</v>
@@ -8466,19 +8552,19 @@
       </c>
       <c r="B72" s="4"/>
       <c r="C72" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="D72" s="4" t="s">
         <v>415</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>416</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>316</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="H72" s="16" t="s">
         <v>197</v>
@@ -8487,7 +8573,7 @@
         <v>191</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K72" s="4">
         <v>10</v>
@@ -8506,19 +8592,19 @@
       </c>
       <c r="B73" s="4"/>
       <c r="C73" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="D73" s="4" t="s">
         <v>418</v>
-      </c>
-      <c r="D73" s="4" t="s">
-        <v>419</v>
       </c>
       <c r="E73" s="4" t="s">
         <v>316</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="H73" s="16" t="s">
         <v>197</v>
@@ -8546,19 +8632,19 @@
       </c>
       <c r="B74" s="19"/>
       <c r="C74" s="19" t="s">
+        <v>420</v>
+      </c>
+      <c r="D74" s="19" t="s">
         <v>421</v>
-      </c>
-      <c r="D74" s="19" t="s">
-        <v>422</v>
       </c>
       <c r="E74" s="19" t="s">
         <v>316</v>
       </c>
       <c r="F74" s="19" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G74" s="19" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H74" s="20" t="s">
         <v>197</v>
@@ -8567,7 +8653,7 @@
         <v>191</v>
       </c>
       <c r="J74" s="19" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K74" s="4">
         <v>13</v>
@@ -8586,19 +8672,19 @@
       </c>
       <c r="B75" s="4"/>
       <c r="C75" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="D75" s="4" t="s">
         <v>424</v>
-      </c>
-      <c r="D75" s="4" t="s">
-        <v>425</v>
       </c>
       <c r="E75" s="4" t="s">
         <v>265</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="H75" s="16" t="s">
         <v>197</v>
@@ -8626,19 +8712,19 @@
       </c>
       <c r="B76" s="14"/>
       <c r="C76" s="14" t="s">
+        <v>426</v>
+      </c>
+      <c r="D76" s="14" t="s">
         <v>427</v>
       </c>
-      <c r="D76" s="14" t="s">
+      <c r="E76" s="14" t="s">
         <v>428</v>
       </c>
-      <c r="E76" s="14" t="s">
+      <c r="F76" s="14" t="s">
+        <v>395</v>
+      </c>
+      <c r="G76" s="14" t="s">
         <v>429</v>
-      </c>
-      <c r="F76" s="14" t="s">
-        <v>396</v>
-      </c>
-      <c r="G76" s="14" t="s">
-        <v>430</v>
       </c>
       <c r="H76" s="15" t="s">
         <v>74</v>
@@ -8659,7 +8745,7 @@
         <v>10</v>
       </c>
       <c r="N76" s="14" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="77" ht="40" customHeight="1" spans="1:14">
@@ -8668,19 +8754,19 @@
       </c>
       <c r="B77" s="4"/>
       <c r="C77" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="G77" s="4" t="s">
         <v>431</v>
-      </c>
-      <c r="D77" s="4" t="s">
-        <v>428</v>
-      </c>
-      <c r="E77" s="4" t="s">
-        <v>429</v>
-      </c>
-      <c r="F77" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="G77" s="4" t="s">
-        <v>432</v>
       </c>
       <c r="H77" s="16" t="s">
         <v>197</v>
@@ -8708,19 +8794,19 @@
       </c>
       <c r="B78" s="4"/>
       <c r="C78" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="D78" s="4" t="s">
         <v>433</v>
       </c>
-      <c r="D78" s="4" t="s">
+      <c r="E78" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="F78" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="G78" s="4" t="s">
         <v>434</v>
-      </c>
-      <c r="E78" s="4" t="s">
-        <v>429</v>
-      </c>
-      <c r="F78" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="G78" s="4" t="s">
-        <v>435</v>
       </c>
       <c r="H78" s="16" t="s">
         <v>197</v>
@@ -8729,7 +8815,7 @@
         <v>191</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="K78" s="4">
         <v>8</v>
@@ -8748,19 +8834,19 @@
       </c>
       <c r="B79" s="4"/>
       <c r="C79" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="D79" s="4" t="s">
         <v>436</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>437</v>
       </c>
       <c r="E79" s="4" t="s">
         <v>283</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="H79" s="16" t="s">
         <v>197</v>
@@ -8788,19 +8874,19 @@
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="D80" s="4" t="s">
         <v>439</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>440</v>
       </c>
       <c r="E80" s="4" t="s">
         <v>283</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="H80" s="4" t="s">
         <v>197</v>
@@ -8809,7 +8895,7 @@
         <v>123</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="K80" s="4">
         <v>5</v>
@@ -8828,19 +8914,19 @@
       </c>
       <c r="B81" s="4"/>
       <c r="C81" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="D81" s="4" t="s">
         <v>442</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>443</v>
       </c>
       <c r="E81" s="4" t="s">
         <v>283</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="H81" s="4" t="s">
         <v>197</v>
@@ -8849,7 +8935,7 @@
         <v>123</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="K81" s="4">
         <v>8</v>
@@ -8868,19 +8954,19 @@
       </c>
       <c r="B82" s="4"/>
       <c r="C82" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="D82" s="4" t="s">
         <v>445</v>
       </c>
-      <c r="D82" s="4" t="s">
+      <c r="E82" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="G82" s="4" t="s">
         <v>446</v>
-      </c>
-      <c r="E82" s="4" t="s">
-        <v>339</v>
-      </c>
-      <c r="F82" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="G82" s="4" t="s">
-        <v>447</v>
       </c>
       <c r="H82" s="4" t="s">
         <v>197</v>
@@ -8889,7 +8975,7 @@
         <v>191</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="K82" s="4">
         <v>8</v>
@@ -8903,8 +8989,8 @@
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1" spans="1:14">
-      <c r="A83" s="32" t="s">
-        <v>448</v>
+      <c r="A83" s="34" t="s">
+        <v>447</v>
       </c>
     </row>
     <row r="84" ht="33" customHeight="1" spans="1:14">
@@ -8913,19 +8999,19 @@
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="D84" s="4" t="s">
         <v>449</v>
       </c>
-      <c r="D84" s="4" t="s">
+      <c r="E84" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="F84" s="4" t="s">
         <v>450</v>
       </c>
-      <c r="E84" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="F84" s="4" t="s">
+      <c r="G84" s="4" t="s">
         <v>451</v>
-      </c>
-      <c r="G84" s="4" t="s">
-        <v>452</v>
       </c>
       <c r="H84" s="4" t="s">
         <v>197</v>
@@ -8934,23 +9020,23 @@
         <v>74</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="K84" s="4" t="s">
         <v>74</v>
       </c>
       <c r="L84" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="M84" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="N84" s="4" t="s">
         <v>453</v>
       </c>
-      <c r="M84" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="N84" s="4" t="s">
-        <v>454</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="29">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A4:N4"/>
@@ -8971,6 +9057,15 @@
     <mergeCell ref="K6:K10"/>
     <mergeCell ref="K12:K17"/>
     <mergeCell ref="K19:K24"/>
+    <mergeCell ref="K26:K27"/>
+    <mergeCell ref="K29:K30"/>
+    <mergeCell ref="K32:K33"/>
+    <mergeCell ref="K35:K37"/>
+    <mergeCell ref="K39:K40"/>
+    <mergeCell ref="K42:K45"/>
+    <mergeCell ref="K47:K51"/>
+    <mergeCell ref="K53:K57"/>
+    <mergeCell ref="K59:K64"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
@@ -9004,12 +9099,12 @@
   <sheetData>
     <row r="1" ht="20.25" customHeight="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1" spans="1:13">
       <c r="A2" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:13">
@@ -9055,7 +9150,7 @@
     </row>
     <row r="4" ht="40" customHeight="1" spans="1:13">
       <c r="A4" s="13" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1" spans="1:13">
@@ -9063,19 +9158,19 @@
         <v>117</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>457</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>458</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>459</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>460</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>121</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G5" s="15" t="s">
         <v>74</v>
@@ -9096,7 +9191,7 @@
         <v>10</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="1:13">
@@ -9104,19 +9199,19 @@
         <v>125</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>463</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>464</v>
-      </c>
       <c r="D6" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G6" s="16" t="s">
         <v>197</v>
@@ -9131,13 +9226,13 @@
         <v>15</v>
       </c>
       <c r="K6" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="M6" s="4" t="s">
         <v>466</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>467</v>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:13">
@@ -9145,19 +9240,19 @@
         <v>125</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>468</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>469</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>470</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="G7" s="16" t="s">
         <v>197</v>
@@ -9166,13 +9261,13 @@
         <v>123</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="J7" s="4">
         <v>8</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L7" s="4" t="s">
         <v>74</v>
@@ -9186,19 +9281,19 @@
         <v>117</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>471</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>472</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" s="14" t="s">
         <v>473</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>474</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>121</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="G8" s="15" t="s">
         <v>74</v>
@@ -9207,7 +9302,7 @@
         <v>123</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="J8" s="14" t="s">
         <v>74</v>
@@ -9227,19 +9322,19 @@
         <v>125</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>476</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>477</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>478</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="G9" s="16" t="s">
         <v>197</v>
@@ -9248,19 +9343,19 @@
         <v>123</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="J9" s="4">
         <v>8</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L9" s="4" t="s">
         <v>74</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1" spans="1:13">
@@ -9268,19 +9363,19 @@
         <v>125</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>481</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>482</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>483</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>197</v>
@@ -9289,19 +9384,19 @@
         <v>123</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="J10" s="4">
         <v>5</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L10" s="4" t="s">
         <v>74</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1" spans="1:13">
@@ -9314,19 +9409,19 @@
         <v>125</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>486</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>487</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>488</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="G12" s="16" t="s">
         <v>197</v>
@@ -9335,13 +9430,13 @@
         <v>123</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="J12" s="4">
         <v>10</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L12" s="4" t="s">
         <v>74</v>
@@ -9355,19 +9450,19 @@
         <v>125</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>490</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>491</v>
-      </c>
       <c r="D13" s="4" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>197</v>
@@ -9376,13 +9471,13 @@
         <v>123</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="J13" s="4">
         <v>8</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>74</v>
@@ -9396,19 +9491,19 @@
         <v>125</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>493</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>494</v>
-      </c>
       <c r="D14" s="4" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="G14" s="16" t="s">
         <v>197</v>
@@ -9417,13 +9512,13 @@
         <v>123</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="J14" s="4">
         <v>10</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L14" s="4" t="s">
         <v>74</v>
@@ -9437,19 +9532,19 @@
         <v>125</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>496</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>497</v>
-      </c>
       <c r="D15" s="4" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="G15" s="16" t="s">
         <v>197</v>
@@ -9458,13 +9553,13 @@
         <v>123</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="J15" s="4">
         <v>8</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L15" s="4" t="s">
         <v>74</v>
@@ -9478,19 +9573,19 @@
         <v>125</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>498</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>499</v>
-      </c>
       <c r="D16" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="G16" s="16" t="s">
         <v>197</v>
@@ -9499,13 +9594,13 @@
         <v>123</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="J16" s="4">
         <v>8</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L16" s="4" t="s">
         <v>74</v>
@@ -9519,19 +9614,19 @@
         <v>125</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>501</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>502</v>
-      </c>
       <c r="D17" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="G17" s="16" t="s">
         <v>197</v>
@@ -9546,7 +9641,7 @@
         <v>13</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L17" s="4" t="s">
         <v>74</v>
@@ -9560,19 +9655,19 @@
         <v>125</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>504</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>505</v>
-      </c>
       <c r="D18" s="4" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="G18" s="16" t="s">
         <v>197</v>
@@ -9581,13 +9676,13 @@
         <v>123</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="J18" s="4">
         <v>13</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L18" s="4" t="s">
         <v>74</v>
@@ -9598,7 +9693,7 @@
     </row>
     <row r="19" ht="96" customHeight="1" spans="1:13">
       <c r="A19" s="17" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:13">
@@ -9606,19 +9701,19 @@
         <v>117</v>
       </c>
       <c r="B20" s="14" t="s">
+        <v>507</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>508</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="D20" s="14" t="s">
         <v>509</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="E20" s="14" t="s">
+        <v>395</v>
+      </c>
+      <c r="F20" s="14" t="s">
         <v>510</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>396</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>511</v>
       </c>
       <c r="G20" s="15" t="s">
         <v>74</v>
@@ -9627,7 +9722,7 @@
         <v>123</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="J20" s="14" t="s">
         <v>74</v>
@@ -9639,7 +9734,7 @@
         <v>10</v>
       </c>
       <c r="M20" s="14" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" spans="1:13">
@@ -9652,19 +9747,19 @@
         <v>125</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>513</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4" t="s">
         <v>514</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>515</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>516</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>197</v>
@@ -9673,13 +9768,13 @@
         <v>123</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="J22" s="4">
         <v>10</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L22" s="4" t="s">
         <v>74</v>
@@ -9727,12 +9822,12 @@
   <sheetData>
     <row r="1" ht="20.25" customHeight="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1" spans="1:13">
       <c r="A2" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:13">
@@ -9778,7 +9873,7 @@
     </row>
     <row r="4" ht="40" customHeight="1" spans="1:13">
       <c r="A4" s="13" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1" spans="1:13">
@@ -9786,19 +9881,19 @@
         <v>117</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>520</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>521</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>522</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>523</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>121</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="G5" s="15" t="s">
         <v>74</v>
@@ -9827,19 +9922,19 @@
         <v>125</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>525</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>526</v>
-      </c>
       <c r="D6" s="4" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="G6" s="16" t="s">
         <v>197</v>
@@ -9854,13 +9949,13 @@
         <v>10</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L6" s="4" t="s">
         <v>74</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:13">
@@ -9868,19 +9963,19 @@
         <v>117</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>528</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>529</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="14" t="s">
         <v>530</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>531</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>121</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>74</v>
@@ -9889,7 +9984,7 @@
         <v>123</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="J7" s="14" t="s">
         <v>74</v>
@@ -9901,7 +9996,7 @@
         <v>10</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1" spans="1:13">
@@ -9909,19 +10004,19 @@
         <v>125</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>534</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>535</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>121</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="G8" s="16" t="s">
         <v>197</v>
@@ -9930,24 +10025,24 @@
         <v>191</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="J8" s="4">
         <v>8</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L8" s="4" t="s">
         <v>74</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1" spans="1:13">
       <c r="A9" s="22" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1" spans="1:13">
@@ -9955,19 +10050,19 @@
         <v>125</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>539</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>540</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>541</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>197</v>
@@ -9976,19 +10071,19 @@
         <v>123</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="J10" s="4">
         <v>13</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L10" s="4" t="s">
         <v>74</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1" spans="1:13">
@@ -9996,19 +10091,19 @@
         <v>117</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>542</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>543</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D11" s="14" t="s">
+        <v>522</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>395</v>
+      </c>
+      <c r="F11" s="14" t="s">
         <v>544</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>523</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>396</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>545</v>
       </c>
       <c r="G11" s="15" t="s">
         <v>74</v>
@@ -10029,7 +10124,7 @@
         <v>10</v>
       </c>
       <c r="M11" s="14" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="12" ht="40" customHeight="1" spans="1:13">
@@ -10037,19 +10132,19 @@
         <v>125</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>547</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>548</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>549</v>
       </c>
       <c r="G12" s="16" t="s">
         <v>197</v>
@@ -10064,13 +10159,13 @@
         <v>10</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L12" s="4" t="s">
         <v>74</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1" spans="1:13">
@@ -10078,19 +10173,19 @@
         <v>125</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>551</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>552</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>553</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>197</v>
@@ -10099,13 +10194,13 @@
         <v>123</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="J13" s="4">
         <v>8</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>74</v>
@@ -10119,19 +10214,19 @@
         <v>117</v>
       </c>
       <c r="B14" s="14" t="s">
+        <v>553</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>554</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D14" s="14" t="s">
+        <v>530</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>395</v>
+      </c>
+      <c r="F14" s="14" t="s">
         <v>555</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>531</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>396</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>556</v>
       </c>
       <c r="G14" s="15" t="s">
         <v>74</v>
@@ -10140,7 +10235,7 @@
         <v>123</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="J14" s="14" t="s">
         <v>74</v>
@@ -10152,7 +10247,7 @@
         <v>10</v>
       </c>
       <c r="M14" s="14" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="15" ht="40" customHeight="1" spans="1:13">
@@ -10160,19 +10255,19 @@
         <v>125</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>558</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>559</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>531</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>560</v>
       </c>
       <c r="G15" s="16" t="s">
         <v>197</v>
@@ -10181,19 +10276,19 @@
         <v>123</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="J15" s="4">
         <v>13</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L15" s="4" t="s">
         <v>74</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:13">
@@ -10201,19 +10296,19 @@
         <v>125</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>562</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>563</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>531</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>396</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>564</v>
       </c>
       <c r="G16" s="16" t="s">
         <v>197</v>
@@ -10222,13 +10317,13 @@
         <v>123</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J16" s="4">
         <v>8</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L16" s="4" t="s">
         <v>74</v>
@@ -10239,7 +10334,7 @@
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:13">
       <c r="A17" s="17" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" spans="1:13">
@@ -10247,19 +10342,19 @@
         <v>125</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>566</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>567</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>531</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>451</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>568</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>197</v>
@@ -10268,13 +10363,13 @@
         <v>123</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="J18" s="4">
         <v>10</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L18" s="4" t="s">
         <v>74</v>
@@ -10323,12 +10418,12 @@
   <sheetData>
     <row r="1" ht="20.25" customHeight="1" spans="1:13">
       <c r="A1" s="1" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1" spans="1:13">
+      <c r="A2" s="23" t="s">
         <v>569</v>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1" spans="1:13">
-      <c r="A2" s="2" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:13">
@@ -10446,7 +10541,7 @@
       <c r="I6" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="16">
         <v>10</v>
       </c>
       <c r="K6" s="4" t="s">
@@ -10487,9 +10582,7 @@
       <c r="I7" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="J7" s="4">
-        <v>10</v>
-      </c>
+      <c r="J7" s="16"/>
       <c r="K7" s="4" t="s">
         <v>583</v>
       </c>
@@ -10528,9 +10621,7 @@
       <c r="I8" s="4" t="s">
         <v>580</v>
       </c>
-      <c r="J8" s="4">
-        <v>8</v>
-      </c>
+      <c r="J8" s="16"/>
       <c r="K8" s="4" t="s">
         <v>578</v>
       </c>
@@ -10564,14 +10655,12 @@
         <v>144</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I9" s="19" t="s">
         <v>575</v>
       </c>
-      <c r="J9" s="4">
-        <v>13</v>
-      </c>
+      <c r="J9" s="16"/>
       <c r="K9" s="4" t="s">
         <v>593</v>
       </c>
@@ -10610,9 +10699,7 @@
       <c r="I10" s="14" t="s">
         <v>575</v>
       </c>
-      <c r="J10" s="14" t="s">
-        <v>74</v>
-      </c>
+      <c r="J10" s="24"/>
       <c r="K10" s="14" t="s">
         <v>74</v>
       </c>
@@ -10651,9 +10738,7 @@
       <c r="I11" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="J11" s="4">
-        <v>8</v>
-      </c>
+      <c r="J11" s="16"/>
       <c r="K11" s="4" t="s">
         <v>583</v>
       </c>
@@ -10692,9 +10777,7 @@
       <c r="I12" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="J12" s="4">
-        <v>5</v>
-      </c>
+      <c r="J12" s="16"/>
       <c r="K12" s="4" t="s">
         <v>583</v>
       </c>
@@ -10733,9 +10816,7 @@
       <c r="I13" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="J13" s="4">
-        <v>10</v>
-      </c>
+      <c r="J13" s="16"/>
       <c r="K13" s="4" t="s">
         <v>578</v>
       </c>
@@ -10774,9 +10855,7 @@
       <c r="I14" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="J14" s="4">
-        <v>13</v>
-      </c>
+      <c r="J14" s="16"/>
       <c r="K14" s="4" t="s">
         <v>578</v>
       </c>
@@ -10815,9 +10894,7 @@
       <c r="I15" s="4" t="s">
         <v>602</v>
       </c>
-      <c r="J15" s="4">
-        <v>10</v>
-      </c>
+      <c r="J15" s="16"/>
       <c r="K15" s="4" t="s">
         <v>578</v>
       </c>
@@ -10856,9 +10933,7 @@
       <c r="I16" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="J16" s="4">
-        <v>8</v>
-      </c>
+      <c r="J16" s="16"/>
       <c r="K16" s="4" t="s">
         <v>578</v>
       </c>
@@ -10897,9 +10972,7 @@
       <c r="I17" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="J17" s="4">
-        <v>8</v>
-      </c>
+      <c r="J17" s="16"/>
       <c r="K17" s="4" t="s">
         <v>578</v>
       </c>
@@ -10938,9 +11011,7 @@
       <c r="I18" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="J18" s="4">
-        <v>10</v>
-      </c>
+      <c r="J18" s="16"/>
       <c r="K18" s="4" t="s">
         <v>578</v>
       </c>
@@ -10979,9 +11050,7 @@
       <c r="I19" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="J19" s="4">
-        <v>8</v>
-      </c>
+      <c r="J19" s="16"/>
       <c r="K19" s="4" t="s">
         <v>578</v>
       </c>
@@ -11020,9 +11089,7 @@
       <c r="I20" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="J20" s="4">
-        <v>8</v>
-      </c>
+      <c r="J20" s="16"/>
       <c r="K20" s="4" t="s">
         <v>578</v>
       </c>
@@ -11061,9 +11128,7 @@
       <c r="I21" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="J21" s="4">
-        <v>8</v>
-      </c>
+      <c r="J21" s="16"/>
       <c r="K21" s="4" t="s">
         <v>578</v>
       </c>
@@ -11102,9 +11167,7 @@
       <c r="I22" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="J22" s="4">
-        <v>8</v>
-      </c>
+      <c r="J22" s="16"/>
       <c r="K22" s="4" t="s">
         <v>578</v>
       </c>
@@ -11143,9 +11206,7 @@
       <c r="I23" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="J23" s="4">
-        <v>8</v>
-      </c>
+      <c r="J23" s="16"/>
       <c r="K23" s="4" t="s">
         <v>578</v>
       </c>
@@ -11184,9 +11245,7 @@
       <c r="I24" s="4" t="s">
         <v>602</v>
       </c>
-      <c r="J24" s="4">
-        <v>10</v>
-      </c>
+      <c r="J24" s="16"/>
       <c r="K24" s="4" t="s">
         <v>578</v>
       </c>
@@ -11225,9 +11284,7 @@
       <c r="I25" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="J25" s="4">
-        <v>13</v>
-      </c>
+      <c r="J25" s="16"/>
       <c r="K25" s="4" t="s">
         <v>583</v>
       </c>
@@ -11266,9 +11323,7 @@
       <c r="I26" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="J26" s="4">
-        <v>15</v>
-      </c>
+      <c r="J26" s="16"/>
       <c r="K26" s="4" t="s">
         <v>583</v>
       </c>
@@ -11280,10 +11335,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A4:M4"/>
+    <mergeCell ref="J6:J26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
@@ -11942,7 +11998,7 @@
         <v>74</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="19" ht="40" customHeight="1" spans="1:13">
@@ -11983,7 +12039,7 @@
         <v>74</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1" spans="1:13">
@@ -12003,7 +12059,7 @@
         <v>121</v>
       </c>
       <c r="F20" s="16" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="G20" s="16" t="s">
         <v>197</v>
@@ -12024,7 +12080,7 @@
         <v>74</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="21" ht="40" customHeight="1" spans="1:13">
@@ -12050,7 +12106,7 @@
         <v>144</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>719</v>
@@ -12342,7 +12398,7 @@
         <v>197</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I29" s="4" t="s">
         <v>693</v>
@@ -12379,7 +12435,7 @@
         <v>703</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F31" s="19" t="s">
         <v>766</v>
@@ -12420,7 +12476,7 @@
         <v>703</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>769</v>
@@ -12461,7 +12517,7 @@
         <v>738</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>772</v>
@@ -12507,7 +12563,7 @@
         <v>685</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>776</v>
@@ -12698,7 +12754,7 @@
       <c r="I6" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="16">
         <v>8</v>
       </c>
       <c r="K6" s="18" t="s">
@@ -12739,9 +12795,7 @@
       <c r="I7" s="4" t="s">
         <v>786</v>
       </c>
-      <c r="J7" s="4">
-        <v>5</v>
-      </c>
+      <c r="J7" s="16"/>
       <c r="K7" s="18" t="s">
         <v>789</v>
       </c>
@@ -12780,9 +12834,7 @@
       <c r="I8" s="4" t="s">
         <v>786</v>
       </c>
-      <c r="J8" s="4">
-        <v>5</v>
-      </c>
+      <c r="J8" s="16"/>
       <c r="K8" s="18" t="s">
         <v>789</v>
       </c>
@@ -12860,7 +12912,7 @@
         <v>191</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J10" s="4">
         <v>13</v>
@@ -12980,7 +13032,7 @@
         <v>144</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I13" s="19" t="s">
         <v>786</v>
@@ -13135,7 +13187,7 @@
         <v>836</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>837</v>
@@ -13176,7 +13228,7 @@
         <v>841</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="16" t="s">
@@ -13215,7 +13267,7 @@
         <v>846</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="16" t="s">
@@ -13254,7 +13306,7 @@
         <v>849</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F20" s="19" t="s">
         <v>850</v>
@@ -13286,7 +13338,7 @@
         <v>125</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>851</v>
@@ -13295,7 +13347,7 @@
         <v>852</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>851</v>
@@ -13336,7 +13388,7 @@
         <v>783</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F22" s="19" t="s">
         <v>855</v>
@@ -13380,7 +13432,7 @@
         <v>859</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F24" s="14" t="s">
         <v>860</v>
@@ -13421,7 +13473,7 @@
         <v>859</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F25" s="19" t="s">
         <v>864</v>
@@ -13462,7 +13514,7 @@
         <v>867</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>868</v>
@@ -13503,7 +13555,7 @@
         <v>867</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F27" s="19" t="s">
         <v>872</v>
@@ -13544,7 +13596,7 @@
         <v>783</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F28" s="14" t="s">
         <v>875</v>
@@ -13585,7 +13637,7 @@
         <v>783</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F29" s="19" t="s">
         <v>879</v>
@@ -13626,7 +13678,7 @@
         <v>800</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F30" s="14" t="s">
         <v>883</v>
@@ -13667,7 +13719,7 @@
         <v>800</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>887</v>
@@ -13695,11 +13747,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="A23:M23"/>
+    <mergeCell ref="J6:J8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
@@ -13970,7 +14023,7 @@
         <v>895</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>913</v>
@@ -14011,7 +14064,7 @@
         <v>895</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>917</v>
@@ -14052,7 +14105,7 @@
         <v>895</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>920</v>
@@ -14093,7 +14146,7 @@
         <v>895</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>922</v>

</xml_diff>

<commit_message>
vault backup: 2026-07-21 11:48:40
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/MVP功能清单.xlsx
+++ b/公司项目/认知作战/文档/MVP功能清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="32400" windowHeight="17820" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="12420" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="说明" sheetId="1" r:id="rId1"/>
@@ -347,8 +347,8 @@
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
-        <color rgb="FF595959"/>
+        <sz val="18"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Calibri"/>
         <charset val="134"/>
       </rPr>
@@ -356,8 +356,8 @@
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
-        <color rgb="FF595959"/>
+        <sz val="18"/>
+        <color rgb="FFFF0000"/>
         <rFont val="Noto Serif CJK SC"/>
         <charset val="134"/>
       </rPr>
@@ -3639,7 +3639,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="45">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -3707,6 +3707,12 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="18"/>
+      <color rgb="FFFF0000"/>
+      <name val="Noto Serif CJK SC"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
@@ -3720,6 +3726,11 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="22"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Noto Serif CJK SC"/>
       <charset val="134"/>
@@ -3728,6 +3739,13 @@
       <b/>
       <sz val="10"/>
       <name val="Noto Serif CJK SC"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -3907,6 +3925,12 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -4261,31 +4285,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="19" fillId="0" borderId="0">
+    <xf numFmtId="43" fontId="22" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="19" fillId="0" borderId="0">
+    <xf numFmtId="44" fontId="22" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="19" fillId="0" borderId="0">
+    <xf numFmtId="9" fontId="22" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="19" fillId="0" borderId="0">
+    <xf numFmtId="41" fontId="22" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="19" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0">
+    <xf numFmtId="42" fontId="22" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
@@ -4294,119 +4306,131 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="3">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="4">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="5">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="4">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="6">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="8">
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="0">
+    <xf numFmtId="0" fontId="34" fillId="13" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="7">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="3" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="39" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="34" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="36" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="37" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="38" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="36" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4478,37 +4502,43 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4521,10 +4551,10 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -4928,65 +4958,65 @@
   </cols>
   <sheetData>
     <row r="1" ht="23.25" customHeight="1" spans="1:2">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:2">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="38" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:2">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="40" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:2">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="40" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:2">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="40" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="39">
+      <c r="B7" s="41">
         <v>46223</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:2">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="40" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:2">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="42" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" ht="55" customHeight="1" spans="1:2">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="40" t="s">
         <v>12</v>
       </c>
     </row>
@@ -4996,7 +5026,7 @@
       </c>
     </row>
     <row r="12" ht="55" customHeight="1" spans="1:2">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="43" t="s">
         <v>14</v>
       </c>
     </row>
@@ -5006,17 +5036,17 @@
       </c>
     </row>
     <row r="14" ht="55" customHeight="1" spans="1:2">
-      <c r="A14" s="38" t="s">
+      <c r="A14" s="40" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:2">
-      <c r="A15" s="40" t="s">
+      <c r="A15" s="42" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" ht="55" customHeight="1" spans="1:2">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="40" t="s">
         <v>18</v>
       </c>
     </row>
@@ -5026,7 +5056,7 @@
       </c>
     </row>
     <row r="18" ht="25" customHeight="1" spans="1:3">
-      <c r="A18" s="41" t="s">
+      <c r="A18" s="43" t="s">
         <v>20</v>
       </c>
     </row>
@@ -5036,20 +5066,20 @@
       </c>
     </row>
     <row r="20" ht="25" customHeight="1" spans="1:3">
-      <c r="A20" s="38" t="s">
+      <c r="A20" s="40" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:3">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="42" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="22" ht="40" customHeight="1" spans="1:3">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="42"/>
+      <c r="C22" s="44"/>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:3">
       <c r="A23" s="21" t="s">
@@ -5057,34 +5087,34 @@
       </c>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:3">
-      <c r="A24" s="38" t="s">
+      <c r="A24" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="38" t="s">
+      <c r="B24" s="40" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:3">
-      <c r="A25" s="38" t="s">
+      <c r="A25" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="38" t="s">
+      <c r="B25" s="40" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:3">
-      <c r="A26" s="38" t="s">
+      <c r="A26" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="38" t="s">
+      <c r="B26" s="40" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:3">
-      <c r="A27" s="38" t="s">
+      <c r="A27" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="38" t="s">
+      <c r="B27" s="40" t="s">
         <v>33</v>
       </c>
       <c r="C27">
@@ -5092,10 +5122,10 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:3">
-      <c r="A28" s="38" t="s">
+      <c r="A28" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="38" t="s">
+      <c r="B28" s="40" t="s">
         <v>35</v>
       </c>
       <c r="C28">
@@ -5103,10 +5133,10 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1" spans="1:3">
-      <c r="A29" s="38" t="s">
+      <c r="A29" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="38" t="s">
+      <c r="B29" s="40" t="s">
         <v>37</v>
       </c>
       <c r="C29">
@@ -5114,10 +5144,10 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:3">
-      <c r="A30" s="38" t="s">
+      <c r="A30" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="B30" s="38" t="s">
+      <c r="B30" s="40" t="s">
         <v>39</v>
       </c>
       <c r="C30">
@@ -5125,10 +5155,10 @@
       </c>
     </row>
     <row r="31" ht="22" customHeight="1" spans="1:3">
-      <c r="A31" s="38" t="s">
+      <c r="A31" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B31" s="38" t="s">
+      <c r="B31" s="40" t="s">
         <v>41</v>
       </c>
       <c r="C31">
@@ -5136,10 +5166,10 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:3">
-      <c r="A32" s="38" t="s">
+      <c r="A32" s="40" t="s">
         <v>42</v>
       </c>
-      <c r="B32" s="38" t="s">
+      <c r="B32" s="40" t="s">
         <v>43</v>
       </c>
       <c r="C32">
@@ -5147,10 +5177,10 @@
       </c>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:2">
-      <c r="A33" s="38" t="s">
+      <c r="A33" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="B33" s="38" t="s">
+      <c r="B33" s="40" t="s">
         <v>45</v>
       </c>
     </row>
@@ -5806,7 +5836,7 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1" spans="1:14">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="25" t="s">
         <v>101</v>
       </c>
     </row>
@@ -5814,7 +5844,7 @@
       <c r="A3" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="26" t="s">
         <v>103</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -5867,7 +5897,7 @@
       <c r="C5" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="27" t="s">
         <v>119</v>
       </c>
       <c r="E5" s="14" t="s">
@@ -5905,7 +5935,7 @@
       <c r="A6" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="28" t="s">
         <v>126</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -5932,7 +5962,7 @@
       <c r="J6" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="K6" s="16">
+      <c r="K6" s="29">
         <v>5</v>
       </c>
       <c r="L6" s="18" t="s">
@@ -5974,7 +6004,7 @@
       <c r="J7" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K7" s="16"/>
+      <c r="K7" s="29"/>
       <c r="L7" s="18" t="s">
         <v>131</v>
       </c>
@@ -6014,7 +6044,7 @@
       <c r="J8" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K8" s="16"/>
+      <c r="K8" s="29"/>
       <c r="L8" s="18" t="s">
         <v>131</v>
       </c>
@@ -6042,7 +6072,7 @@
       <c r="F9" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="G9" s="28" t="s">
         <v>143</v>
       </c>
       <c r="H9" s="16" t="s">
@@ -6054,7 +6084,7 @@
       <c r="J9" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K9" s="16"/>
+      <c r="K9" s="29"/>
       <c r="L9" s="18" t="s">
         <v>131</v>
       </c>
@@ -6094,7 +6124,7 @@
       <c r="J10" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K10" s="16"/>
+      <c r="K10" s="29"/>
       <c r="L10" s="18" t="s">
         <v>131</v>
       </c>
@@ -6111,7 +6141,7 @@
       <c r="C11" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="27" t="s">
         <v>150</v>
       </c>
       <c r="E11" s="14" t="s">
@@ -6147,7 +6177,7 @@
       <c r="A12" t="s">
         <v>125</v>
       </c>
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="30" t="s">
         <v>154</v>
       </c>
       <c r="C12" t="s">
@@ -6188,7 +6218,7 @@
       <c r="A13" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="30"/>
+      <c r="B13" s="31"/>
       <c r="C13" t="s">
         <v>160</v>
       </c>
@@ -6228,7 +6258,7 @@
       <c r="A14" t="s">
         <v>125</v>
       </c>
-      <c r="B14" s="30"/>
+      <c r="B14" s="31"/>
       <c r="C14" t="s">
         <v>165</v>
       </c>
@@ -6265,7 +6295,7 @@
       <c r="A15" t="s">
         <v>125</v>
       </c>
-      <c r="B15" s="30"/>
+      <c r="B15" s="31"/>
       <c r="C15" t="s">
         <v>169</v>
       </c>
@@ -6302,7 +6332,7 @@
       <c r="A16" t="s">
         <v>125</v>
       </c>
-      <c r="B16" s="30"/>
+      <c r="B16" s="31"/>
       <c r="C16" t="s">
         <v>173</v>
       </c>
@@ -6339,7 +6369,7 @@
       <c r="A17" t="s">
         <v>125</v>
       </c>
-      <c r="B17" s="30"/>
+      <c r="B17" s="31"/>
       <c r="C17" t="s">
         <v>177</v>
       </c>
@@ -6352,7 +6382,7 @@
       <c r="F17" t="s">
         <v>121</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="G17" s="28" t="s">
         <v>179</v>
       </c>
       <c r="H17" t="s">
@@ -6421,7 +6451,7 @@
       <c r="A19" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="28" t="s">
         <v>187</v>
       </c>
       <c r="C19" s="4" t="s">
@@ -6448,7 +6478,7 @@
       <c r="J19" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K19" s="16">
+      <c r="K19" s="29">
         <v>7</v>
       </c>
       <c r="L19" s="18" t="s">
@@ -6490,7 +6520,7 @@
       <c r="J20" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="K20" s="16"/>
+      <c r="K20" s="29"/>
       <c r="L20" s="18" t="s">
         <v>192</v>
       </c>
@@ -6530,7 +6560,7 @@
       <c r="J21" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="K21" s="16"/>
+      <c r="K21" s="29"/>
       <c r="L21" s="18" t="s">
         <v>192</v>
       </c>
@@ -6570,7 +6600,7 @@
       <c r="J22" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="K22" s="16"/>
+      <c r="K22" s="29"/>
       <c r="L22" s="18" t="s">
         <v>192</v>
       </c>
@@ -6610,7 +6640,7 @@
       <c r="J23" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="K23" s="16"/>
+      <c r="K23" s="29"/>
       <c r="L23" s="18" t="s">
         <v>192</v>
       </c>
@@ -6650,7 +6680,7 @@
       <c r="J24" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="K24" s="16"/>
+      <c r="K24" s="29"/>
       <c r="L24" s="18" t="s">
         <v>192</v>
       </c>
@@ -6734,7 +6764,7 @@
       <c r="J26" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="K26" s="16">
+      <c r="K26" s="29">
         <v>5</v>
       </c>
       <c r="L26" s="18" t="s">
@@ -6770,13 +6800,13 @@
       <c r="H27" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="I27" s="31" t="s">
+      <c r="I27" s="32" t="s">
         <v>123</v>
       </c>
       <c r="J27" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="K27" s="16"/>
+      <c r="K27" s="29"/>
       <c r="L27" s="18" t="s">
         <v>192</v>
       </c>
@@ -6833,7 +6863,7 @@
       <c r="A29" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B29" s="27" t="s">
+      <c r="B29" s="28" t="s">
         <v>154</v>
       </c>
       <c r="C29" s="4" t="s">
@@ -6860,7 +6890,7 @@
       <c r="J29" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="K29" s="16">
+      <c r="K29" s="29">
         <v>7</v>
       </c>
       <c r="L29" t="s">
@@ -6902,7 +6932,7 @@
       <c r="J30" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="K30" s="16"/>
+      <c r="K30" s="29"/>
       <c r="L30" t="s">
         <v>158</v>
       </c>
@@ -6959,7 +6989,7 @@
       <c r="A32" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B32" s="27" t="s">
+      <c r="B32" s="28" t="s">
         <v>187</v>
       </c>
       <c r="C32" s="4" t="s">
@@ -6986,7 +7016,7 @@
       <c r="J32" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K32" s="16">
+      <c r="K32" s="29">
         <v>14</v>
       </c>
       <c r="L32" s="18" t="s">
@@ -7028,7 +7058,7 @@
       <c r="J33" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K33" s="16"/>
+      <c r="K33" s="29"/>
       <c r="L33" s="18" t="s">
         <v>131</v>
       </c>
@@ -7112,7 +7142,7 @@
       <c r="J35" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="K35" s="16">
+      <c r="K35" s="29">
         <v>5</v>
       </c>
       <c r="L35" s="18" t="s">
@@ -7154,7 +7184,7 @@
       <c r="J36" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="K36" s="16"/>
+      <c r="K36" s="29"/>
       <c r="L36" s="18" t="s">
         <v>192</v>
       </c>
@@ -7194,7 +7224,7 @@
       <c r="J37" s="19" t="s">
         <v>273</v>
       </c>
-      <c r="K37" s="16"/>
+      <c r="K37" s="29"/>
       <c r="L37" s="18" t="s">
         <v>192</v>
       </c>
@@ -7251,7 +7281,7 @@
       <c r="A39" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="27" t="s">
+      <c r="B39" s="28" t="s">
         <v>286</v>
       </c>
       <c r="C39" s="4" t="s">
@@ -7278,7 +7308,7 @@
       <c r="J39" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="K39" s="16">
+      <c r="K39" s="29">
         <v>5</v>
       </c>
       <c r="L39" s="18" t="s">
@@ -7320,7 +7350,7 @@
       <c r="J40" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="K40" s="16"/>
+      <c r="K40" s="29"/>
       <c r="L40" s="18" t="s">
         <v>8</v>
       </c>
@@ -7404,7 +7434,7 @@
       <c r="J42" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="K42" s="16">
+      <c r="K42" s="29">
         <v>7</v>
       </c>
       <c r="L42" s="18" t="s">
@@ -7446,7 +7476,7 @@
       <c r="J43" s="4" t="s">
         <v>300</v>
       </c>
-      <c r="K43" s="16"/>
+      <c r="K43" s="29"/>
       <c r="L43" s="18" t="s">
         <v>131</v>
       </c>
@@ -7486,7 +7516,7 @@
       <c r="J44" s="19" t="s">
         <v>300</v>
       </c>
-      <c r="K44" s="16"/>
+      <c r="K44" s="29"/>
       <c r="L44" s="18" t="s">
         <v>131</v>
       </c>
@@ -7526,7 +7556,7 @@
       <c r="J45" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="K45" s="16"/>
+      <c r="K45" s="29"/>
       <c r="L45" s="18" t="s">
         <v>131</v>
       </c>
@@ -7583,7 +7613,7 @@
       <c r="A47" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B47" s="27" t="s">
+      <c r="B47" s="28" t="s">
         <v>187</v>
       </c>
       <c r="C47" s="4" t="s">
@@ -7610,7 +7640,7 @@
       <c r="J47" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="K47" s="16">
+      <c r="K47" s="29">
         <v>7</v>
       </c>
       <c r="L47" s="18" t="s">
@@ -7652,7 +7682,7 @@
       <c r="J48" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="K48" s="16"/>
+      <c r="K48" s="29"/>
       <c r="L48" s="18" t="s">
         <v>192</v>
       </c>
@@ -7692,7 +7722,7 @@
       <c r="J49" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="K49" s="16"/>
+      <c r="K49" s="29"/>
       <c r="L49" s="18" t="s">
         <v>192</v>
       </c>
@@ -7732,7 +7762,7 @@
       <c r="J50" s="19" t="s">
         <v>319</v>
       </c>
-      <c r="K50" s="16"/>
+      <c r="K50" s="29"/>
       <c r="L50" s="18" t="s">
         <v>192</v>
       </c>
@@ -7772,7 +7802,7 @@
       <c r="J51" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="K51" s="16"/>
+      <c r="K51" s="29"/>
       <c r="L51" s="18" t="s">
         <v>192</v>
       </c>
@@ -7856,7 +7886,7 @@
       <c r="J53" s="19" t="s">
         <v>340</v>
       </c>
-      <c r="K53" s="16">
+      <c r="K53" s="29">
         <v>5</v>
       </c>
       <c r="L53" s="18" t="s">
@@ -7898,7 +7928,7 @@
       <c r="J54" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="K54" s="16"/>
+      <c r="K54" s="29"/>
       <c r="L54" s="18" t="s">
         <v>8</v>
       </c>
@@ -7938,7 +7968,7 @@
       <c r="J55" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="K55" s="16"/>
+      <c r="K55" s="29"/>
       <c r="L55" s="18" t="s">
         <v>8</v>
       </c>
@@ -7978,7 +8008,7 @@
       <c r="J56" s="4" t="s">
         <v>357</v>
       </c>
-      <c r="K56" s="16"/>
+      <c r="K56" s="29"/>
       <c r="L56" s="18" t="s">
         <v>8</v>
       </c>
@@ -8018,7 +8048,7 @@
       <c r="J57" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="K57" s="16"/>
+      <c r="K57" s="29"/>
       <c r="L57" s="18" t="s">
         <v>8</v>
       </c>
@@ -8043,7 +8073,7 @@
       <c r="E58" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="F58" s="14" t="s">
+      <c r="F58" s="33" t="s">
         <v>229</v>
       </c>
       <c r="G58" s="15" t="s">
@@ -8128,7 +8158,7 @@
       <c r="F60" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="G60" s="32" t="s">
+      <c r="G60" s="34" t="s">
         <v>375</v>
       </c>
       <c r="H60" s="20" t="s">
@@ -8302,7 +8332,7 @@
       </c>
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:14">
-      <c r="A65" s="33" t="s">
+      <c r="A65" s="35" t="s">
         <v>392</v>
       </c>
     </row>
@@ -8989,7 +9019,7 @@
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1" spans="1:14">
-      <c r="A83" s="34" t="s">
+      <c r="A83" s="36" t="s">
         <v>447</v>
       </c>
     </row>
@@ -9055,8 +9085,8 @@
     <mergeCell ref="B53:B57"/>
     <mergeCell ref="B59:B64"/>
     <mergeCell ref="K6:K10"/>
-    <mergeCell ref="K12:K17"/>
-    <mergeCell ref="K19:K24"/>
+    <mergeCell ref="K12:K16"/>
+    <mergeCell ref="K19:K23"/>
     <mergeCell ref="K26:K27"/>
     <mergeCell ref="K29:K30"/>
     <mergeCell ref="K32:K33"/>

</xml_diff>